<commit_message>
Make corrections on ordering and shipping processes
Direct influence of vax order on backlog and supply rate on inventory have been eliminated
</commit_message>
<xml_diff>
--- a/Data/national-puskesmas-VSC.xlsx
+++ b/Data/national-puskesmas-VSC.xlsx
@@ -8,21 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fc1fb\Models\Vax SC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575BD2FD-F166-4BB1-9CBC-1B315DFC557E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E45BB7B3-DF0C-44EB-9031-953C85E874D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="18000" windowHeight="8670" activeTab="2" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="1" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
   </bookViews>
   <sheets>
     <sheet name="NationalOffice" sheetId="1" r:id="rId1"/>
     <sheet name="ProvincialPublicHealth" sheetId="2" r:id="rId2"/>
-    <sheet name="Puskesmas" sheetId="3" r:id="rId3"/>
+    <sheet name="DistrictHealthOffice" sheetId="4" r:id="rId3"/>
+    <sheet name="Puskesmas" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="36">
   <si>
     <t>Name</t>
   </si>
@@ -36,12 +50,6 @@
     <t>Warehouse</t>
   </si>
   <si>
-    <t>DKI Jakarta</t>
-  </si>
-  <si>
-    <t>East Kalimantan</t>
-  </si>
-  <si>
     <t>North Kalimantan</t>
   </si>
   <si>
@@ -57,47 +65,92 @@
     <t>Type</t>
   </si>
   <si>
-    <t>PHPapua</t>
-  </si>
-  <si>
-    <t>PHEastKalimantan</t>
-  </si>
-  <si>
-    <t>PHWestPapua</t>
-  </si>
-  <si>
-    <t>PHNorthKalimantan</t>
-  </si>
-  <si>
     <t>Provincial Health Office</t>
   </si>
   <si>
-    <t>PuskesmasKebayoranLama</t>
-  </si>
-  <si>
-    <t>PuskesmasSamarindaKota</t>
-  </si>
-  <si>
-    <t>PuskesmasTarakanKota</t>
-  </si>
-  <si>
-    <t>PuskesmasJayapuraKota</t>
-  </si>
-  <si>
-    <t>PuskesmasManokwari</t>
-  </si>
-  <si>
     <t>BioFarma</t>
   </si>
   <si>
     <t>Upstream Connection</t>
+  </si>
+  <si>
+    <t>PHOPapua</t>
+  </si>
+  <si>
+    <t>PHOWestPapua</t>
+  </si>
+  <si>
+    <t>PHONorthKalimantan</t>
+  </si>
+  <si>
+    <t>District Health Office</t>
+  </si>
+  <si>
+    <t>Yapen</t>
+  </si>
+  <si>
+    <t>BiakNumfor</t>
+  </si>
+  <si>
+    <t>Kaimana</t>
+  </si>
+  <si>
+    <t>TelukWondama</t>
+  </si>
+  <si>
+    <t>Malinau</t>
+  </si>
+  <si>
+    <t>Bulungan</t>
+  </si>
+  <si>
+    <t>Wooi</t>
+  </si>
+  <si>
+    <t>Windesi</t>
+  </si>
+  <si>
+    <t>Yomdori</t>
+  </si>
+  <si>
+    <t>Orkeri</t>
+  </si>
+  <si>
+    <t>Tanusan</t>
+  </si>
+  <si>
+    <t>Kambala</t>
+  </si>
+  <si>
+    <t>Roswar</t>
+  </si>
+  <si>
+    <t>Wasior</t>
+  </si>
+  <si>
+    <t>Sesua</t>
+  </si>
+  <si>
+    <t>Bunyu</t>
+  </si>
+  <si>
+    <t>Salimbatu</t>
+  </si>
+  <si>
+    <t>LongSule</t>
+  </si>
+  <si>
+    <t>Annual Demand</t>
+  </si>
+  <si>
+    <t>Initial Demand</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -232,8 +285,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -413,8 +484,44 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC1F0C8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAF2D0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAE9F8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0E6F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE2D5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7C7AC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -529,6 +636,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -574,8 +696,59 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="18" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="18" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="18" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="18" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="18" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -951,18 +1124,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31AE70DF-A7F5-4EBA-9A4E-6625684456F1}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -970,10 +1143,13 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -983,6 +1159,10 @@
       </c>
       <c r="D2">
         <v>107.6045</v>
+      </c>
+      <c r="E2">
+        <f>SUM(ProvincialPublicHealth!F2:F4)</f>
+        <v>8642</v>
       </c>
     </row>
   </sheetData>
@@ -992,19 +1172,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB85C89-820F-4524-AF6D-187344255E48}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1013,75 +1194,73 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2">
-        <v>-2.6028701129999998</v>
+        <v>9</v>
+      </c>
+      <c r="C2" s="2">
+        <v>-2.6025074110039998</v>
       </c>
       <c r="D2">
-        <v>140.6734347</v>
+        <v>140.67348730942601</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="F2">
+        <f>SUM(DistrictHealthOffice!F2:F3)</f>
+        <v>2346</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3">
-        <v>-0.71735368200000005</v>
+        <v>9</v>
+      </c>
+      <c r="C3" s="2">
+        <v>-0.92318704230664395</v>
       </c>
       <c r="D3">
-        <v>134.01607970000001</v>
+        <v>134.03438844232801</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <f>SUM(DistrictHealthOffice!F4:F5)</f>
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4">
-        <v>-0.46881378699999998</v>
+        <v>9</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2.8328995471436702</v>
       </c>
       <c r="D4">
-        <v>117.13919989999999</v>
+        <v>117.39359407772</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5">
-        <v>2.8496995329999999</v>
-      </c>
-      <c r="D5">
-        <v>117.3667038</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
+        <v>10</v>
+      </c>
+      <c r="F4">
+        <f>SUM(DistrictHealthOffice!F6:F7)</f>
+        <v>4980</v>
       </c>
     </row>
   </sheetData>
@@ -1090,20 +1269,183 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D745374B-C969-4E87-BEE9-45241CCB8CDB}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="5" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1">
+        <v>-1.8422904609478199</v>
+      </c>
+      <c r="D2">
+        <v>136.238107390989</v>
+      </c>
+      <c r="E2" t="str">
+        <f>ProvincialPublicHealth!A2</f>
+        <v>PHOPapua</v>
+      </c>
+      <c r="F2">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2">
+        <v>-1.17429952681732</v>
+      </c>
+      <c r="D3">
+        <v>136.07705652966999</v>
+      </c>
+      <c r="E3" t="str">
+        <f>ProvincialPublicHealth!A2</f>
+        <v>PHOPapua</v>
+      </c>
+      <c r="F3">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3">
+        <v>-3.64051869331414</v>
+      </c>
+      <c r="D4">
+        <v>133.74154486024901</v>
+      </c>
+      <c r="E4" t="str">
+        <f>ProvincialPublicHealth!A3</f>
+        <v>PHOWestPapua</v>
+      </c>
+      <c r="F4">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="4">
+        <v>-2.8153222293189</v>
+      </c>
+      <c r="D5">
+        <v>134.53693615007199</v>
+      </c>
+      <c r="E5" t="str">
+        <f>ProvincialPublicHealth!A3</f>
+        <v>PHOWestPapua</v>
+      </c>
+      <c r="F5">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="5">
+        <v>3.6177392015440901</v>
+      </c>
+      <c r="D6">
+        <v>116.608687764956</v>
+      </c>
+      <c r="E6" t="str">
+        <f>ProvincialPublicHealth!A4</f>
+        <v>PHONorthKalimantan</v>
+      </c>
+      <c r="F6">
+        <v>1824</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="7">
+        <v>2.8468313498968398</v>
+      </c>
+      <c r="D7">
+        <v>117.38749377154799</v>
+      </c>
+      <c r="E7" t="str">
+        <f>ProvincialPublicHealth!A4</f>
+        <v>PHONorthKalimantan</v>
+      </c>
+      <c r="F7">
+        <v>3156</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{098AA237-CD4F-4868-9842-2B0C8D95453B}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1112,92 +1454,305 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>16</v>
-      </c>
       <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>-6.238105</v>
+        <v>5</v>
+      </c>
+      <c r="C2" s="8">
+        <v>-1.61064751969144</v>
       </c>
       <c r="D2">
-        <v>106.777916</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>17</v>
+        <v>135.44274443639199</v>
+      </c>
+      <c r="E2" t="str">
+        <f>DistrictHealthOffice!A2</f>
+        <v>Yapen</v>
+      </c>
+      <c r="F2" s="20">
+        <v>660</v>
+      </c>
+      <c r="G2" s="14">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3">
-        <v>-0.50299799999999995</v>
+      <c r="C3" s="8">
+        <v>-1.6366618939606701</v>
       </c>
       <c r="D3">
-        <v>117.153278</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>18</v>
+        <v>135.913922963788</v>
+      </c>
+      <c r="E3" t="str">
+        <f>DistrictHealthOffice!A2</f>
+        <v>Yapen</v>
+      </c>
+      <c r="F3" s="20">
+        <v>660</v>
+      </c>
+      <c r="G3" s="14">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="9">
+        <v>-1.04458743699844</v>
+      </c>
+      <c r="D4">
+        <v>135.86399250532699</v>
+      </c>
+      <c r="E4" t="str">
+        <f>DistrictHealthOffice!A3</f>
+        <v>BiakNumfor</v>
+      </c>
+      <c r="F4" s="21">
+        <v>748</v>
+      </c>
+      <c r="G4" s="15">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="9">
+        <v>-0.95816914533692499</v>
+      </c>
+      <c r="D5">
+        <v>134.91975310065101</v>
+      </c>
+      <c r="E5" t="str">
+        <f>DistrictHealthOffice!A3</f>
+        <v>BiakNumfor</v>
+      </c>
+      <c r="F5" s="21">
+        <v>748</v>
+      </c>
+      <c r="G5" s="15">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="C4">
-        <v>3.3009770000000001</v>
-      </c>
-      <c r="D4">
-        <v>117.597931</v>
-      </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>-2.5338229999999999</v>
-      </c>
-      <c r="D5">
-        <v>140.71806000000001</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>-0.86199400000000004</v>
+      <c r="C6" s="10">
+        <v>-3.0808659690697602</v>
       </c>
       <c r="D6">
-        <v>134.06250600000001</v>
-      </c>
-      <c r="E6" t="s">
-        <v>13</v>
+        <v>133.664687738232</v>
+      </c>
+      <c r="E6" t="str">
+        <f>DistrictHealthOffice!A4</f>
+        <v>Kaimana</v>
+      </c>
+      <c r="F6" s="16">
+        <v>138</v>
+      </c>
+      <c r="G6" s="16">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="10">
+        <v>-3.6201589116883701</v>
+      </c>
+      <c r="D7">
+        <v>133.43101497844799</v>
+      </c>
+      <c r="E7" t="str">
+        <f>DistrictHealthOffice!A4</f>
+        <v>Kaimana</v>
+      </c>
+      <c r="F7" s="16">
+        <v>138</v>
+      </c>
+      <c r="G7" s="16">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="11">
+        <v>-2.0606722996972402</v>
+      </c>
+      <c r="D8">
+        <v>134.35274004669199</v>
+      </c>
+      <c r="E8" t="str">
+        <f>DistrictHealthOffice!A5</f>
+        <v>TelukWondama</v>
+      </c>
+      <c r="F8" s="17">
+        <v>306</v>
+      </c>
+      <c r="G8" s="17">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="11">
+        <v>-2.70027216068081</v>
+      </c>
+      <c r="D9">
+        <v>134.50994578377899</v>
+      </c>
+      <c r="E9" t="str">
+        <f>DistrictHealthOffice!A5</f>
+        <v>TelukWondama</v>
+      </c>
+      <c r="F9" s="17">
+        <v>306</v>
+      </c>
+      <c r="G9" s="17">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="12">
+        <v>1.5334396419363501</v>
+      </c>
+      <c r="D10">
+        <v>115.698051380062</v>
+      </c>
+      <c r="E10" t="str">
+        <f>DistrictHealthOffice!A6</f>
+        <v>Malinau</v>
+      </c>
+      <c r="F10" s="18">
+        <v>759</v>
+      </c>
+      <c r="G10" s="18">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="12">
+        <v>3.4811981002066199</v>
+      </c>
+      <c r="D11">
+        <v>116.659518928121</v>
+      </c>
+      <c r="E11" t="str">
+        <f>DistrictHealthOffice!A6</f>
+        <v>Malinau</v>
+      </c>
+      <c r="F11" s="18">
+        <v>759</v>
+      </c>
+      <c r="G11" s="18">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="13">
+        <v>3.4947019699173798</v>
+      </c>
+      <c r="D12">
+        <v>117.860873683788</v>
+      </c>
+      <c r="E12" t="str">
+        <f>DistrictHealthOffice!A7</f>
+        <v>Bulungan</v>
+      </c>
+      <c r="F12" s="19">
+        <v>1499</v>
+      </c>
+      <c r="G12" s="19">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="13">
+        <v>2.9558984580186198</v>
+      </c>
+      <c r="D13">
+        <v>117.348328497341</v>
+      </c>
+      <c r="E13" t="str">
+        <f>DistrictHealthOffice!A7</f>
+        <v>Bulungan</v>
+      </c>
+      <c r="F13" s="19">
+        <v>1499</v>
+      </c>
+      <c r="G13" s="19">
+        <v>1578</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Import the DRC case study data
</commit_message>
<xml_diff>
--- a/Data/national-puskesmas-VSC.xlsx
+++ b/Data/national-puskesmas-VSC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fc1fb\Models\Vax SC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E45BB7B3-DF0C-44EB-9031-953C85E874D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7DE0893-951D-49A7-94B3-DBBD62C275A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="1" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
   </bookViews>
   <sheets>
     <sheet name="NationalOffice" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="52">
   <si>
     <t>Name</t>
   </si>
@@ -50,15 +50,6 @@
     <t>Warehouse</t>
   </si>
   <si>
-    <t>North Kalimantan</t>
-  </si>
-  <si>
-    <t>Papua</t>
-  </si>
-  <si>
-    <t>West Papua</t>
-  </si>
-  <si>
     <t>Province</t>
   </si>
   <si>
@@ -68,89 +59,146 @@
     <t>Provincial Health Office</t>
   </si>
   <si>
-    <t>BioFarma</t>
-  </si>
-  <si>
     <t>Upstream Connection</t>
   </si>
   <si>
-    <t>PHOPapua</t>
-  </si>
-  <si>
-    <t>PHOWestPapua</t>
-  </si>
-  <si>
-    <t>PHONorthKalimantan</t>
-  </si>
-  <si>
-    <t>District Health Office</t>
-  </si>
-  <si>
-    <t>Yapen</t>
-  </si>
-  <si>
-    <t>BiakNumfor</t>
-  </si>
-  <si>
-    <t>Kaimana</t>
-  </si>
-  <si>
-    <t>TelukWondama</t>
-  </si>
-  <si>
-    <t>Malinau</t>
-  </si>
-  <si>
-    <t>Bulungan</t>
-  </si>
-  <si>
-    <t>Wooi</t>
-  </si>
-  <si>
-    <t>Windesi</t>
-  </si>
-  <si>
-    <t>Yomdori</t>
-  </si>
-  <si>
-    <t>Orkeri</t>
-  </si>
-  <si>
-    <t>Tanusan</t>
-  </si>
-  <si>
-    <t>Kambala</t>
-  </si>
-  <si>
-    <t>Roswar</t>
-  </si>
-  <si>
-    <t>Wasior</t>
-  </si>
-  <si>
-    <t>Sesua</t>
-  </si>
-  <si>
-    <t>Bunyu</t>
-  </si>
-  <si>
-    <t>Salimbatu</t>
-  </si>
-  <si>
-    <t>LongSule</t>
-  </si>
-  <si>
     <t>Annual Demand</t>
   </si>
   <si>
     <t>Initial Demand</t>
+  </si>
+  <si>
+    <t>Mbandaka</t>
+  </si>
+  <si>
+    <t>Basankusu</t>
+  </si>
+  <si>
+    <t>Bikoro</t>
+  </si>
+  <si>
+    <t>Bolenge_s</t>
+  </si>
+  <si>
+    <t>Bolenge_l</t>
+  </si>
+  <si>
+    <t>Bolomba</t>
+  </si>
+  <si>
+    <t>Bomongo</t>
+  </si>
+  <si>
+    <t>Djombo</t>
+  </si>
+  <si>
+    <t>Iboko</t>
+  </si>
+  <si>
+    <t>Ingende</t>
+  </si>
+  <si>
+    <t>Irebu</t>
+  </si>
+  <si>
+    <t>Lilanga Bobangi</t>
+  </si>
+  <si>
+    <t>Lolanga Mampoko</t>
+  </si>
+  <si>
+    <t>Lotumbe</t>
+  </si>
+  <si>
+    <t>Lukolela</t>
+  </si>
+  <si>
+    <t>Makanza</t>
+  </si>
+  <si>
+    <t>Monieka</t>
+  </si>
+  <si>
+    <t>Ntondo</t>
+  </si>
+  <si>
+    <t>Wangata</t>
+  </si>
+  <si>
+    <t>Equateur</t>
+  </si>
+  <si>
+    <t>Health Zone</t>
+  </si>
+  <si>
+    <t>PHOEquateur</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>HZMbandaka</t>
+  </si>
+  <si>
+    <t>HZBasankusu</t>
+  </si>
+  <si>
+    <t>HZBikoro</t>
+  </si>
+  <si>
+    <t>HZBolenge_s</t>
+  </si>
+  <si>
+    <t>HZBolenge_l</t>
+  </si>
+  <si>
+    <t>HZBolomba</t>
+  </si>
+  <si>
+    <t>HZBomongo</t>
+  </si>
+  <si>
+    <t>HZDjombo</t>
+  </si>
+  <si>
+    <t>HZIboko</t>
+  </si>
+  <si>
+    <t>HZIngende</t>
+  </si>
+  <si>
+    <t>HZIrebu</t>
+  </si>
+  <si>
+    <t>HZLilanga Bobangi</t>
+  </si>
+  <si>
+    <t>HZLolanga Mampoko</t>
+  </si>
+  <si>
+    <t>HZLotumbe</t>
+  </si>
+  <si>
+    <t>HZLukolela</t>
+  </si>
+  <si>
+    <t>HZMakanza</t>
+  </si>
+  <si>
+    <t>HZMonieka</t>
+  </si>
+  <si>
+    <t>HZNtondo</t>
+  </si>
+  <si>
+    <t>HZWangata</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -291,20 +339,8 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="39">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -484,44 +520,8 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC1F0C8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDAF2D0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDAE9F8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC0E6F5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFBE2D5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF7C7AC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -636,21 +636,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -696,59 +681,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="2" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="18" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="18" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="18" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="18" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="18" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1128,6 +1063,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1135,7 +1071,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1144,25 +1080,25 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2">
-        <v>-6.8975999999999997</v>
-      </c>
-      <c r="D2">
-        <v>107.6045</v>
+      <c r="C2" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="D2" s="1">
+        <v>18.391999999999999</v>
       </c>
       <c r="E2">
         <f>SUM(ProvincialPublicHealth!F2:F4)</f>
-        <v>8642</v>
+        <v>135414.99986458503</v>
       </c>
     </row>
   </sheetData>
@@ -1172,7 +1108,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB85C89-820F-4524-AF6D-187344255E48}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -1185,7 +1121,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1194,73 +1130,31 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="2">
-        <v>-2.6025074110039998</v>
-      </c>
-      <c r="D2">
-        <v>140.67348730942601</v>
+        <v>6</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="D2" s="1">
+        <v>18.391999999999999</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="F2">
-        <f>SUM(DistrictHealthOffice!F2:F3)</f>
-        <v>2346</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2">
-        <v>-0.92318704230664395</v>
-      </c>
-      <c r="D3">
-        <v>134.03438844232801</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3">
-        <f>SUM(DistrictHealthOffice!F4:F5)</f>
-        <v>1316</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="5">
-        <v>2.8328995471436702</v>
-      </c>
-      <c r="D4">
-        <v>117.39359407772</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4">
-        <f>SUM(DistrictHealthOffice!F6:F7)</f>
-        <v>4980</v>
+        <f>SUM(DistrictHealthOffice!F2:F20)</f>
+        <v>135414.99986458503</v>
       </c>
     </row>
   </sheetData>
@@ -1270,20 +1164,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D745374B-C969-4E87-BEE9-45241CCB8CDB}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="5" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1292,137 +1187,410 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="D2" s="1">
+        <v>18.391999999999999</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="1">
+        <v>8610.3048173800016</v>
+      </c>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.92100000000000004</v>
+      </c>
+      <c r="D3" s="1">
+        <v>19.881</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="1">
+        <v>15304.90717126</v>
+      </c>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1">
-        <v>-1.8422904609478199</v>
-      </c>
-      <c r="D2">
-        <v>136.238107390989</v>
-      </c>
-      <c r="E2" t="str">
-        <f>ProvincialPublicHealth!A2</f>
-        <v>PHOPapua</v>
-      </c>
-      <c r="F2">
-        <v>1348</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="2">
-        <v>-1.17429952681732</v>
-      </c>
-      <c r="D3">
-        <v>136.07705652966999</v>
-      </c>
-      <c r="E3" t="str">
-        <f>ProvincialPublicHealth!A2</f>
-        <v>PHOPapua</v>
-      </c>
-      <c r="F3">
-        <v>998</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="3">
-        <v>-3.64051869331414</v>
-      </c>
-      <c r="D4">
-        <v>133.74154486024901</v>
-      </c>
-      <c r="E4" t="str">
-        <f>ProvincialPublicHealth!A3</f>
-        <v>PHOWestPapua</v>
-      </c>
-      <c r="F4">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>19</v>
+        <v>30</v>
+      </c>
+      <c r="C4" s="1">
+        <v>-0.46600000000000003</v>
+      </c>
+      <c r="D4" s="1">
+        <v>18.231999999999999</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="1">
+        <v>9126.6690245499994</v>
+      </c>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4">
-        <v>-2.8153222293189</v>
-      </c>
-      <c r="D5">
-        <v>134.53693615007199</v>
-      </c>
-      <c r="E5" t="str">
-        <f>ProvincialPublicHealth!A3</f>
-        <v>PHOWestPapua</v>
-      </c>
-      <c r="F5">
-        <v>812</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>20</v>
+        <v>30</v>
+      </c>
+      <c r="C5" s="1">
+        <v>-0.20300000000000001</v>
+      </c>
+      <c r="D5" s="1">
+        <v>18.038</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="1">
+        <v>280.11906275500002</v>
+      </c>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="5">
-        <v>3.6177392015440901</v>
-      </c>
-      <c r="D6">
-        <v>116.608687764956</v>
-      </c>
-      <c r="E6" t="str">
-        <f>ProvincialPublicHealth!A4</f>
-        <v>PHONorthKalimantan</v>
-      </c>
-      <c r="F6">
-        <v>1824</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>21</v>
+        <v>30</v>
+      </c>
+      <c r="C6" s="1">
+        <v>-0.11700000000000001</v>
+      </c>
+      <c r="D6" s="1">
+        <v>18.297000000000001</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="1">
+        <v>4805.3036487400004</v>
+      </c>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="7">
-        <v>2.8468313498968398</v>
-      </c>
-      <c r="D7">
-        <v>117.38749377154799</v>
-      </c>
-      <c r="E7" t="str">
-        <f>ProvincialPublicHealth!A4</f>
-        <v>PHONorthKalimantan</v>
-      </c>
-      <c r="F7">
-        <v>3156</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.35099999999999998</v>
+      </c>
+      <c r="D7" s="1">
+        <v>19.091000000000001</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="1">
+        <v>16407.648796805002</v>
+      </c>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1.5149999999999999</v>
+      </c>
+      <c r="D8" s="1">
+        <v>18.442</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="1">
+        <v>6537.5688907900003</v>
+      </c>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1.369</v>
+      </c>
+      <c r="D9" s="1">
+        <v>20.341000000000001</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="1">
+        <v>6854.878329145</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="1">
+        <v>-0.94799999999999995</v>
+      </c>
+      <c r="D10" s="1">
+        <v>18.606000000000002</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="1">
+        <v>6122.6511017000003</v>
+      </c>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="1">
+        <v>-0.44900000000000001</v>
+      </c>
+      <c r="D11" s="1">
+        <v>18.832999999999998</v>
+      </c>
+      <c r="E11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="1">
+        <v>9024.4946154300014</v>
+      </c>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1">
+        <v>-0.74399999999999999</v>
+      </c>
+      <c r="D12" s="1">
+        <v>17.663</v>
+      </c>
+      <c r="E12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="1">
+        <v>2155.6533748050001</v>
+      </c>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="D13" s="1">
+        <v>17.978000000000002</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="1">
+        <v>4905.8897753250003</v>
+      </c>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.86499999999999999</v>
+      </c>
+      <c r="D14" s="1">
+        <v>18.713000000000001</v>
+      </c>
+      <c r="E14" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="1">
+        <v>5484.9879603749996</v>
+      </c>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="1">
+        <v>-0.68200000000000005</v>
+      </c>
+      <c r="D15" s="1">
+        <v>19.683</v>
+      </c>
+      <c r="E15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="1">
+        <v>6403.4319375599998</v>
+      </c>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="1">
+        <v>-1.423</v>
+      </c>
+      <c r="D16" s="1">
+        <v>17.143999999999998</v>
+      </c>
+      <c r="E16" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" s="1">
+        <v>8500.9836108050004</v>
+      </c>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1.5449999999999999</v>
+      </c>
+      <c r="D17" s="1">
+        <v>19.071999999999999</v>
+      </c>
+      <c r="E17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" s="1">
+        <v>7278.1341614450002</v>
+      </c>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="1">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="D18" s="1">
+        <v>20.032</v>
+      </c>
+      <c r="E18" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="1">
+        <v>4833.8913802199995</v>
+      </c>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="1">
+        <v>-1.0740000000000001</v>
+      </c>
+      <c r="D19" s="1">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="E19" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" s="1">
+        <v>3899.8299910850001</v>
+      </c>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="1">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="D20" s="1">
+        <v>18.231000000000002</v>
+      </c>
+      <c r="E20" t="s">
+        <v>31</v>
+      </c>
+      <c r="F20" s="1">
+        <v>8877.6522144099999</v>
+      </c>
+      <c r="G20" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1431,7 +1599,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{098AA237-CD4F-4868-9842-2B0C8D95453B}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
@@ -1440,12 +1608,12 @@
     <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1454,301 +1622,469 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="D2" s="1">
+        <v>18.391999999999999</v>
+      </c>
+      <c r="E2" t="str">
+        <f t="shared" ref="E2:E6" si="0">_xlfn.CONCAT("HZ",A2)</f>
+        <v>HZMbandaka</v>
+      </c>
+      <c r="F2" s="1">
+        <v>8610.3048173800016</v>
+      </c>
+      <c r="G2" s="1">
+        <v>8610.3048173800016</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.92100000000000004</v>
+      </c>
+      <c r="D3" s="1">
+        <v>19.881</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" si="0"/>
+        <v>HZBasankusu</v>
+      </c>
+      <c r="F3" s="1">
+        <v>15304.90717126</v>
+      </c>
+      <c r="G3" s="1">
+        <v>15304.90717126</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1">
+        <v>-0.46600000000000003</v>
+      </c>
+      <c r="D4" s="1">
+        <v>18.231999999999999</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>HZBikoro</v>
+      </c>
+      <c r="F4" s="1">
+        <v>9126.6690245499994</v>
+      </c>
+      <c r="G4" s="1">
+        <v>9126.6690245499994</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="1">
+        <v>-0.20300000000000001</v>
+      </c>
+      <c r="D5" s="1">
+        <v>18.038</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>HZBolenge_s</v>
+      </c>
+      <c r="F5" s="1">
+        <v>280.11906275500002</v>
+      </c>
+      <c r="G5" s="1">
+        <v>280.11906275500002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="1">
+        <v>-0.11700000000000001</v>
+      </c>
+      <c r="D6" s="1">
+        <v>18.297000000000001</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>HZBolenge_l</v>
+      </c>
+      <c r="F6" s="1">
+        <v>4805.3036487400004</v>
+      </c>
+      <c r="G6" s="1">
+        <v>4805.3036487400004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.35099999999999998</v>
+      </c>
+      <c r="D7" s="1">
+        <v>19.091000000000001</v>
+      </c>
+      <c r="E7" t="str">
+        <f>_xlfn.CONCAT("HZ",A7)</f>
+        <v>HZBolomba</v>
+      </c>
+      <c r="F7" s="1">
+        <v>16407.648796805002</v>
+      </c>
+      <c r="G7" s="1">
+        <v>16407.648796805002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1.5149999999999999</v>
+      </c>
+      <c r="D8" s="1">
+        <v>18.442</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" ref="E8:E20" si="1">_xlfn.CONCAT("HZ",A8)</f>
+        <v>HZBomongo</v>
+      </c>
+      <c r="F8" s="1">
+        <v>6537.5688907900003</v>
+      </c>
+      <c r="G8" s="1">
+        <v>6537.5688907900003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1.369</v>
+      </c>
+      <c r="D9" s="1">
+        <v>20.341000000000001</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="1"/>
+        <v>HZDjombo</v>
+      </c>
+      <c r="F9" s="1">
+        <v>6854.878329145</v>
+      </c>
+      <c r="G9" s="1">
+        <v>6854.878329145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="1">
+        <v>-0.94799999999999995</v>
+      </c>
+      <c r="D10" s="1">
+        <v>18.606000000000002</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="1"/>
+        <v>HZIboko</v>
+      </c>
+      <c r="F10" s="1">
+        <v>6122.6511017000003</v>
+      </c>
+      <c r="G10" s="1">
+        <v>6122.6511017000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="1">
+        <v>-0.44900000000000001</v>
+      </c>
+      <c r="D11" s="1">
+        <v>18.832999999999998</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="1"/>
+        <v>HZIngende</v>
+      </c>
+      <c r="F11" s="1">
+        <v>9024.4946154300014</v>
+      </c>
+      <c r="G11" s="1">
+        <v>9024.4946154300014</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="1">
+        <v>-0.74399999999999999</v>
+      </c>
+      <c r="D12" s="1">
+        <v>17.663</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="1"/>
+        <v>HZIrebu</v>
+      </c>
+      <c r="F12" s="1">
+        <v>2155.6533748050001</v>
+      </c>
+      <c r="G12" s="1">
+        <v>2155.6533748050001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="D13" s="1">
+        <v>17.978000000000002</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="1"/>
+        <v>HZLilanga Bobangi</v>
+      </c>
+      <c r="F13" s="1">
+        <v>4905.8897753250003</v>
+      </c>
+      <c r="G13" s="1">
+        <v>4905.8897753250003</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="8">
-        <v>-1.61064751969144</v>
-      </c>
-      <c r="D2">
-        <v>135.44274443639199</v>
-      </c>
-      <c r="E2" t="str">
-        <f>DistrictHealthOffice!A2</f>
-        <v>Yapen</v>
-      </c>
-      <c r="F2" s="20">
-        <v>660</v>
-      </c>
-      <c r="G2" s="14">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.86499999999999999</v>
+      </c>
+      <c r="D14" s="1">
+        <v>18.713000000000001</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="1"/>
+        <v>HZLolanga Mampoko</v>
+      </c>
+      <c r="F14" s="1">
+        <v>5484.9879603749996</v>
+      </c>
+      <c r="G14" s="1">
+        <v>5484.9879603749996</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="8">
-        <v>-1.6366618939606701</v>
-      </c>
-      <c r="D3">
-        <v>135.913922963788</v>
-      </c>
-      <c r="E3" t="str">
-        <f>DistrictHealthOffice!A2</f>
-        <v>Yapen</v>
-      </c>
-      <c r="F3" s="20">
-        <v>660</v>
-      </c>
-      <c r="G3" s="14">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="1">
+        <v>-0.68200000000000005</v>
+      </c>
+      <c r="D15" s="1">
+        <v>19.683</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="1"/>
+        <v>HZLotumbe</v>
+      </c>
+      <c r="F15" s="1">
+        <v>6403.4319375599998</v>
+      </c>
+      <c r="G15" s="1">
+        <v>6403.4319375599998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="9">
-        <v>-1.04458743699844</v>
-      </c>
-      <c r="D4">
-        <v>135.86399250532699</v>
-      </c>
-      <c r="E4" t="str">
-        <f>DistrictHealthOffice!A3</f>
-        <v>BiakNumfor</v>
-      </c>
-      <c r="F4" s="21">
-        <v>748</v>
-      </c>
-      <c r="G4" s="15">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="1">
+        <v>-1.423</v>
+      </c>
+      <c r="D16" s="1">
+        <v>17.143999999999998</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="1"/>
+        <v>HZLukolela</v>
+      </c>
+      <c r="F16" s="1">
+        <v>8500.9836108050004</v>
+      </c>
+      <c r="G16" s="1">
+        <v>8500.9836108050004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="9">
-        <v>-0.95816914533692499</v>
-      </c>
-      <c r="D5">
-        <v>134.91975310065101</v>
-      </c>
-      <c r="E5" t="str">
-        <f>DistrictHealthOffice!A3</f>
-        <v>BiakNumfor</v>
-      </c>
-      <c r="F5" s="21">
-        <v>748</v>
-      </c>
-      <c r="G5" s="15">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1.5449999999999999</v>
+      </c>
+      <c r="D17" s="1">
+        <v>19.071999999999999</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="1"/>
+        <v>HZMakanza</v>
+      </c>
+      <c r="F17" s="1">
+        <v>7278.1341614450002</v>
+      </c>
+      <c r="G17" s="1">
+        <v>7278.1341614450002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="10">
-        <v>-3.0808659690697602</v>
-      </c>
-      <c r="D6">
-        <v>133.664687738232</v>
-      </c>
-      <c r="E6" t="str">
-        <f>DistrictHealthOffice!A4</f>
-        <v>Kaimana</v>
-      </c>
-      <c r="F6" s="16">
-        <v>138</v>
-      </c>
-      <c r="G6" s="16">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="B18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="1">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="D18" s="1">
+        <v>20.032</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="1"/>
+        <v>HZMonieka</v>
+      </c>
+      <c r="F18" s="1">
+        <v>4833.8913802199995</v>
+      </c>
+      <c r="G18" s="1">
+        <v>4833.8913802199995</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="10">
-        <v>-3.6201589116883701</v>
-      </c>
-      <c r="D7">
-        <v>133.43101497844799</v>
-      </c>
-      <c r="E7" t="str">
-        <f>DistrictHealthOffice!A4</f>
-        <v>Kaimana</v>
-      </c>
-      <c r="F7" s="16">
-        <v>138</v>
-      </c>
-      <c r="G7" s="16">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="B19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="1">
+        <v>-1.0740000000000001</v>
+      </c>
+      <c r="D19" s="1">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="1"/>
+        <v>HZNtondo</v>
+      </c>
+      <c r="F19" s="1">
+        <v>3899.8299910850001</v>
+      </c>
+      <c r="G19" s="1">
+        <v>3899.8299910850001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="11">
-        <v>-2.0606722996972402</v>
-      </c>
-      <c r="D8">
-        <v>134.35274004669199</v>
-      </c>
-      <c r="E8" t="str">
-        <f>DistrictHealthOffice!A5</f>
-        <v>TelukWondama</v>
-      </c>
-      <c r="F8" s="17">
-        <v>306</v>
-      </c>
-      <c r="G8" s="17">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="B20" t="s">
         <v>29</v>
       </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="11">
-        <v>-2.70027216068081</v>
-      </c>
-      <c r="D9">
-        <v>134.50994578377899</v>
-      </c>
-      <c r="E9" t="str">
-        <f>DistrictHealthOffice!A5</f>
-        <v>TelukWondama</v>
-      </c>
-      <c r="F9" s="17">
-        <v>306</v>
-      </c>
-      <c r="G9" s="17">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="12">
-        <v>1.5334396419363501</v>
-      </c>
-      <c r="D10">
-        <v>115.698051380062</v>
-      </c>
-      <c r="E10" t="str">
-        <f>DistrictHealthOffice!A6</f>
-        <v>Malinau</v>
-      </c>
-      <c r="F10" s="18">
-        <v>759</v>
-      </c>
-      <c r="G10" s="18">
-        <v>912</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="12">
-        <v>3.4811981002066199</v>
-      </c>
-      <c r="D11">
-        <v>116.659518928121</v>
-      </c>
-      <c r="E11" t="str">
-        <f>DistrictHealthOffice!A6</f>
-        <v>Malinau</v>
-      </c>
-      <c r="F11" s="18">
-        <v>759</v>
-      </c>
-      <c r="G11" s="18">
-        <v>912</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="13">
-        <v>3.4947019699173798</v>
-      </c>
-      <c r="D12">
-        <v>117.860873683788</v>
-      </c>
-      <c r="E12" t="str">
-        <f>DistrictHealthOffice!A7</f>
-        <v>Bulungan</v>
-      </c>
-      <c r="F12" s="19">
-        <v>1499</v>
-      </c>
-      <c r="G12" s="19">
-        <v>1578</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="13">
-        <v>2.9558984580186198</v>
-      </c>
-      <c r="D13">
-        <v>117.348328497341</v>
-      </c>
-      <c r="E13" t="str">
-        <f>DistrictHealthOffice!A7</f>
-        <v>Bulungan</v>
-      </c>
-      <c r="F13" s="19">
-        <v>1499</v>
-      </c>
-      <c r="G13" s="19">
-        <v>1578</v>
+      <c r="C20" s="1">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="D20" s="1">
+        <v>18.231000000000002</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="1"/>
+        <v>HZWangata</v>
+      </c>
+      <c r="F20" s="1">
+        <v>8877.6522144099999</v>
+      </c>
+      <c r="G20" s="1">
+        <v>8877.6522144099999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Change the data to high demand
</commit_message>
<xml_diff>
--- a/Data/national-puskesmas-VSC.xlsx
+++ b/Data/national-puskesmas-VSC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fc1fb\Models\Vax SC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7DE0893-951D-49A7-94B3-DBBD62C275A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DCA8F2-AF63-49AF-87C3-ED50FB88BE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
   </bookViews>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="E2">
         <f>SUM(ProvincialPublicHealth!F2:F4)</f>
-        <v>135414.99986458503</v>
+        <v>1824999.9981750008</v>
       </c>
     </row>
   </sheetData>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F2">
         <f>SUM(DistrictHealthOffice!F2:F20)</f>
-        <v>135414.99986458503</v>
+        <v>1824999.9981750008</v>
       </c>
     </row>
   </sheetData>
@@ -1210,7 +1210,8 @@
         <v>31</v>
       </c>
       <c r="F2" s="1">
-        <v>8610.3048173800016</v>
+        <f>Puskesmas!G2</f>
+        <v>116041.84390000002</v>
       </c>
       <c r="G2" s="1"/>
     </row>
@@ -1231,7 +1232,8 @@
         <v>31</v>
       </c>
       <c r="F3" s="1">
-        <v>15304.90717126</v>
+        <f>Puskesmas!G3</f>
+        <v>206265.59529999999</v>
       </c>
       <c r="G3" s="1"/>
     </row>
@@ -1252,7 +1254,8 @@
         <v>31</v>
       </c>
       <c r="F4" s="1">
-        <v>9126.6690245499994</v>
+        <f>Puskesmas!G4</f>
+        <v>123000.93025</v>
       </c>
       <c r="G4" s="1"/>
     </row>
@@ -1273,7 +1276,8 @@
         <v>31</v>
       </c>
       <c r="F5" s="1">
-        <v>280.11906275500002</v>
+        <f>Puskesmas!G5</f>
+        <v>3775.1895250000002</v>
       </c>
       <c r="G5" s="1"/>
     </row>
@@ -1294,7 +1298,8 @@
         <v>31</v>
       </c>
       <c r="F6" s="1">
-        <v>4805.3036487400004</v>
+        <f>Puskesmas!G6</f>
+        <v>64761.504700000005</v>
       </c>
       <c r="G6" s="1"/>
     </row>
@@ -1315,7 +1320,8 @@
         <v>31</v>
       </c>
       <c r="F7" s="1">
-        <v>16407.648796805002</v>
+        <f>Puskesmas!G7</f>
+        <v>221127.34227500003</v>
       </c>
       <c r="G7" s="1"/>
     </row>
@@ -1336,7 +1342,8 @@
         <v>31</v>
       </c>
       <c r="F8" s="1">
-        <v>6537.5688907900003</v>
+        <f>Puskesmas!G8</f>
+        <v>88107.397450000004</v>
       </c>
       <c r="G8" s="1"/>
     </row>
@@ -1357,7 +1364,8 @@
         <v>31</v>
       </c>
       <c r="F9" s="1">
-        <v>6854.878329145</v>
+        <f>Puskesmas!G9</f>
+        <v>92383.804974999992</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -1378,7 +1386,8 @@
         <v>31</v>
       </c>
       <c r="F10" s="1">
-        <v>6122.6511017000003</v>
+        <f>Puskesmas!G10</f>
+        <v>82515.513500000001</v>
       </c>
       <c r="G10" s="1"/>
     </row>
@@ -1399,7 +1408,8 @@
         <v>31</v>
       </c>
       <c r="F11" s="1">
-        <v>9024.4946154300014</v>
+        <f>Puskesmas!G11</f>
+        <v>121623.91665000003</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1420,7 +1430,8 @@
         <v>31</v>
       </c>
       <c r="F12" s="1">
-        <v>2155.6533748050001</v>
+        <f>Puskesmas!G12</f>
+        <v>29051.932274999999</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1441,7 +1452,8 @@
         <v>31</v>
       </c>
       <c r="F13" s="1">
-        <v>4905.8897753250003</v>
+        <f>Puskesmas!G13</f>
+        <v>66117.112875000006</v>
       </c>
       <c r="G13" s="1"/>
     </row>
@@ -1462,7 +1474,8 @@
         <v>31</v>
       </c>
       <c r="F14" s="1">
-        <v>5484.9879603749996</v>
+        <f>Puskesmas!G14</f>
+        <v>73921.670624999999</v>
       </c>
       <c r="G14" s="1"/>
     </row>
@@ -1483,7 +1496,8 @@
         <v>31</v>
       </c>
       <c r="F15" s="1">
-        <v>6403.4319375599998</v>
+        <f>Puskesmas!G15</f>
+        <v>86299.621799999994</v>
       </c>
       <c r="G15" s="1"/>
     </row>
@@ -1504,7 +1518,8 @@
         <v>31</v>
       </c>
       <c r="F16" s="1">
-        <v>8500.9836108050004</v>
+        <f>Puskesmas!G16</f>
+        <v>114568.512275</v>
       </c>
       <c r="G16" s="1"/>
     </row>
@@ -1525,7 +1540,8 @@
         <v>31</v>
       </c>
       <c r="F17" s="1">
-        <v>7278.1341614450002</v>
+        <f>Puskesmas!G17</f>
+        <v>98088.06147500001</v>
       </c>
       <c r="G17" s="1"/>
     </row>
@@ -1546,7 +1562,8 @@
         <v>31</v>
       </c>
       <c r="F18" s="1">
-        <v>4833.8913802199995</v>
+        <f>Puskesmas!G18</f>
+        <v>65146.784099999997</v>
       </c>
       <c r="G18" s="1"/>
     </row>
@@ -1567,7 +1584,8 @@
         <v>31</v>
       </c>
       <c r="F19" s="1">
-        <v>3899.8299910850001</v>
+        <f>Puskesmas!G19</f>
+        <v>52558.355675000006</v>
       </c>
       <c r="G19" s="1"/>
     </row>
@@ -1588,7 +1606,8 @@
         <v>31</v>
       </c>
       <c r="F20" s="1">
-        <v>8877.6522144099999</v>
+        <f>Puskesmas!G20</f>
+        <v>119644.90854999999</v>
       </c>
       <c r="G20" s="1"/>
     </row>
@@ -1649,10 +1668,10 @@
         <v>HZMbandaka</v>
       </c>
       <c r="F2" s="1">
-        <v>8610.3048173800016</v>
+        <v>116041.84390000002</v>
       </c>
       <c r="G2" s="1">
-        <v>8610.3048173800016</v>
+        <v>116041.84390000002</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1673,10 +1692,10 @@
         <v>HZBasankusu</v>
       </c>
       <c r="F3" s="1">
-        <v>15304.90717126</v>
+        <v>206265.59529999999</v>
       </c>
       <c r="G3" s="1">
-        <v>15304.90717126</v>
+        <v>206265.59529999999</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1697,10 +1716,10 @@
         <v>HZBikoro</v>
       </c>
       <c r="F4" s="1">
-        <v>9126.6690245499994</v>
+        <v>123000.93025</v>
       </c>
       <c r="G4" s="1">
-        <v>9126.6690245499994</v>
+        <v>123000.93025</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1721,10 +1740,10 @@
         <v>HZBolenge_s</v>
       </c>
       <c r="F5" s="1">
-        <v>280.11906275500002</v>
+        <v>3775.1895250000002</v>
       </c>
       <c r="G5" s="1">
-        <v>280.11906275500002</v>
+        <v>3775.1895250000002</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1745,10 +1764,10 @@
         <v>HZBolenge_l</v>
       </c>
       <c r="F6" s="1">
-        <v>4805.3036487400004</v>
+        <v>64761.504700000005</v>
       </c>
       <c r="G6" s="1">
-        <v>4805.3036487400004</v>
+        <v>64761.504700000005</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1769,10 +1788,10 @@
         <v>HZBolomba</v>
       </c>
       <c r="F7" s="1">
-        <v>16407.648796805002</v>
+        <v>221127.34227500003</v>
       </c>
       <c r="G7" s="1">
-        <v>16407.648796805002</v>
+        <v>221127.34227500003</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1793,10 +1812,10 @@
         <v>HZBomongo</v>
       </c>
       <c r="F8" s="1">
-        <v>6537.5688907900003</v>
+        <v>88107.397450000004</v>
       </c>
       <c r="G8" s="1">
-        <v>6537.5688907900003</v>
+        <v>88107.397450000004</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1817,10 +1836,10 @@
         <v>HZDjombo</v>
       </c>
       <c r="F9" s="1">
-        <v>6854.878329145</v>
+        <v>92383.804974999992</v>
       </c>
       <c r="G9" s="1">
-        <v>6854.878329145</v>
+        <v>92383.804974999992</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1841,10 +1860,10 @@
         <v>HZIboko</v>
       </c>
       <c r="F10" s="1">
-        <v>6122.6511017000003</v>
+        <v>82515.513500000001</v>
       </c>
       <c r="G10" s="1">
-        <v>6122.6511017000003</v>
+        <v>82515.513500000001</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1865,10 +1884,10 @@
         <v>HZIngende</v>
       </c>
       <c r="F11" s="1">
-        <v>9024.4946154300014</v>
+        <v>121623.91665000003</v>
       </c>
       <c r="G11" s="1">
-        <v>9024.4946154300014</v>
+        <v>121623.91665000003</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1889,10 +1908,10 @@
         <v>HZIrebu</v>
       </c>
       <c r="F12" s="1">
-        <v>2155.6533748050001</v>
+        <v>29051.932274999999</v>
       </c>
       <c r="G12" s="1">
-        <v>2155.6533748050001</v>
+        <v>29051.932274999999</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1913,10 +1932,10 @@
         <v>HZLilanga Bobangi</v>
       </c>
       <c r="F13" s="1">
-        <v>4905.8897753250003</v>
+        <v>66117.112875000006</v>
       </c>
       <c r="G13" s="1">
-        <v>4905.8897753250003</v>
+        <v>66117.112875000006</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1937,10 +1956,10 @@
         <v>HZLolanga Mampoko</v>
       </c>
       <c r="F14" s="1">
-        <v>5484.9879603749996</v>
+        <v>73921.670624999999</v>
       </c>
       <c r="G14" s="1">
-        <v>5484.9879603749996</v>
+        <v>73921.670624999999</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1961,10 +1980,10 @@
         <v>HZLotumbe</v>
       </c>
       <c r="F15" s="1">
-        <v>6403.4319375599998</v>
+        <v>86299.621799999994</v>
       </c>
       <c r="G15" s="1">
-        <v>6403.4319375599998</v>
+        <v>86299.621799999994</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1985,10 +2004,10 @@
         <v>HZLukolela</v>
       </c>
       <c r="F16" s="1">
-        <v>8500.9836108050004</v>
+        <v>114568.512275</v>
       </c>
       <c r="G16" s="1">
-        <v>8500.9836108050004</v>
+        <v>114568.512275</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2009,10 +2028,10 @@
         <v>HZMakanza</v>
       </c>
       <c r="F17" s="1">
-        <v>7278.1341614450002</v>
+        <v>98088.06147500001</v>
       </c>
       <c r="G17" s="1">
-        <v>7278.1341614450002</v>
+        <v>98088.06147500001</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -2033,10 +2052,10 @@
         <v>HZMonieka</v>
       </c>
       <c r="F18" s="1">
-        <v>4833.8913802199995</v>
+        <v>65146.784099999997</v>
       </c>
       <c r="G18" s="1">
-        <v>4833.8913802199995</v>
+        <v>65146.784099999997</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2057,10 +2076,10 @@
         <v>HZNtondo</v>
       </c>
       <c r="F19" s="1">
-        <v>3899.8299910850001</v>
+        <v>52558.355675000006</v>
       </c>
       <c r="G19" s="1">
-        <v>3899.8299910850001</v>
+        <v>52558.355675000006</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -2081,10 +2100,10 @@
         <v>HZWangata</v>
       </c>
       <c r="F20" s="1">
-        <v>8877.6522144099999</v>
+        <v>119644.90854999999</v>
       </c>
       <c r="G20" s="1">
-        <v>8877.6522144099999</v>
+        <v>119644.90854999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modify the health zone coordinates
The coordinates of health zones have been changed to reflect the reality
</commit_message>
<xml_diff>
--- a/Data/national-puskesmas-VSC.xlsx
+++ b/Data/national-puskesmas-VSC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fc1fb\Models\Vax SC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DCA8F2-AF63-49AF-87C3-ED50FB88BE78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97917454-86B0-44A7-B611-6211CBC78A71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="3" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
   </bookViews>
   <sheets>
     <sheet name="NationalOffice" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="50">
   <si>
     <t>Name</t>
   </si>
@@ -77,12 +77,6 @@
     <t>Bikoro</t>
   </si>
   <si>
-    <t>Bolenge_s</t>
-  </si>
-  <si>
-    <t>Bolenge_l</t>
-  </si>
-  <si>
     <t>Bolomba</t>
   </si>
   <si>
@@ -146,12 +140,6 @@
     <t>HZBikoro</t>
   </si>
   <si>
-    <t>HZBolenge_s</t>
-  </si>
-  <si>
-    <t>HZBolenge_l</t>
-  </si>
-  <si>
     <t>HZBolomba</t>
   </si>
   <si>
@@ -192,6 +180,12 @@
   </si>
   <si>
     <t>HZWangata</t>
+  </si>
+  <si>
+    <t>HZBolenge</t>
+  </si>
+  <si>
+    <t>Bolenge</t>
   </si>
 </sst>
 </file>
@@ -1085,20 +1079,20 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="1">
-        <v>0.22</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>18.391999999999999</v>
+        <v>18.264500000000002</v>
       </c>
       <c r="E2">
         <f>SUM(ProvincialPublicHealth!F2:F4)</f>
-        <v>1824999.9981750008</v>
+        <v>1889761.5028750007</v>
       </c>
     </row>
   </sheetData>
@@ -1138,23 +1132,23 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="1">
-        <v>0.22</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>18.391999999999999</v>
+        <v>18.264500000000002</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F2">
-        <f>SUM(DistrictHealthOffice!F2:F20)</f>
-        <v>1824999.9981750008</v>
+        <f>SUM(DistrictHealthOffice!F2:F19)</f>
+        <v>1889761.5028750007</v>
       </c>
     </row>
   </sheetData>
@@ -1164,7 +1158,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D745374B-C969-4E87-BEE9-45241CCB8CDB}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -1195,19 +1189,19 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C2" s="1">
-        <v>0.22</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>18.391999999999999</v>
+        <v>18.264500000000002</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F2" s="1">
         <f>Puskesmas!G2</f>
@@ -1217,19 +1211,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C3" s="1">
-        <v>0.92100000000000004</v>
+        <v>1.2185999999999999</v>
       </c>
       <c r="D3" s="1">
-        <v>19.881</v>
+        <v>19.7912</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F3" s="1">
         <f>Puskesmas!G3</f>
@@ -1239,19 +1233,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C4" s="1">
-        <v>-0.46600000000000003</v>
+        <v>-0.72570000000000001</v>
       </c>
       <c r="D4" s="1">
-        <v>18.231999999999999</v>
+        <v>18.124600000000001</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F4" s="1">
         <f>Puskesmas!G4</f>
@@ -1261,355 +1255,333 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C5" s="1">
-        <v>-0.20300000000000001</v>
+        <v>1.8699999999999999E-3</v>
       </c>
       <c r="D5" s="1">
-        <v>18.038</v>
+        <v>18.210999999999999</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F5" s="1">
         <f>Puskesmas!G5</f>
-        <v>3775.1895250000002</v>
+        <v>133298.198925</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C6" s="1">
-        <v>-0.11700000000000001</v>
+        <v>0.35349999999999998</v>
       </c>
       <c r="D6" s="1">
-        <v>18.297000000000001</v>
+        <v>19.222999999999999</v>
       </c>
       <c r="E6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F6" s="1">
         <f>Puskesmas!G6</f>
-        <v>64761.504700000005</v>
+        <v>221127.34227500003</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C7" s="1">
-        <v>0.35099999999999998</v>
+        <v>1.38</v>
       </c>
       <c r="D7" s="1">
-        <v>19.091000000000001</v>
+        <v>18.3506</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F7" s="1">
         <f>Puskesmas!G7</f>
-        <v>221127.34227500003</v>
+        <v>88107.397450000004</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" s="1">
-        <v>1.5149999999999999</v>
+        <v>1.3486</v>
       </c>
       <c r="D8" s="1">
-        <v>18.442</v>
+        <v>20.382899999999999</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F8" s="1">
         <f>Puskesmas!G8</f>
-        <v>88107.397450000004</v>
+        <v>92383.804974999992</v>
       </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C9" s="1">
-        <v>1.369</v>
+        <v>-1.1132</v>
       </c>
       <c r="D9" s="1">
-        <v>20.341000000000001</v>
+        <v>18.5334</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F9" s="1">
         <f>Puskesmas!G9</f>
-        <v>92383.804974999992</v>
+        <v>82515.513500000001</v>
       </c>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C10" s="1">
-        <v>-0.94799999999999995</v>
+        <v>-0.30859999999999999</v>
       </c>
       <c r="D10" s="1">
-        <v>18.606000000000002</v>
+        <v>18.965199999999999</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F10" s="1">
         <f>Puskesmas!G10</f>
-        <v>82515.513500000001</v>
+        <v>121623.91665000003</v>
       </c>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" s="1">
-        <v>-0.44900000000000001</v>
+        <v>-0.61309999999999998</v>
       </c>
       <c r="D11" s="1">
-        <v>18.832999999999998</v>
+        <v>17.740200000000002</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F11" s="1">
         <f>Puskesmas!G11</f>
-        <v>121623.91665000003</v>
+        <v>29051.932274999999</v>
       </c>
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C12" s="1">
-        <v>-0.74399999999999999</v>
+        <v>-0.44059999999999999</v>
       </c>
       <c r="D12" s="1">
-        <v>17.663</v>
+        <v>17.7424</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F12" s="1">
         <f>Puskesmas!G12</f>
-        <v>29051.932274999999</v>
+        <v>66117.112875000006</v>
       </c>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C13" s="1">
-        <v>0.18</v>
+        <v>0.86180000000000001</v>
       </c>
       <c r="D13" s="1">
-        <v>17.978000000000002</v>
+        <v>18.6755</v>
       </c>
       <c r="E13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F13" s="1">
         <f>Puskesmas!G13</f>
-        <v>66117.112875000006</v>
+        <v>73921.670624999999</v>
       </c>
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C14" s="1">
-        <v>0.86499999999999999</v>
+        <v>-0.52459999999999996</v>
       </c>
       <c r="D14" s="1">
-        <v>18.713000000000001</v>
+        <v>19.425599999999999</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F14" s="1">
         <f>Puskesmas!G14</f>
-        <v>73921.670624999999</v>
+        <v>86299.621799999994</v>
       </c>
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C15" s="1">
-        <v>-0.68200000000000005</v>
+        <v>-1.0618000000000001</v>
       </c>
       <c r="D15" s="1">
-        <v>19.683</v>
+        <v>17.177399999999999</v>
       </c>
       <c r="E15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F15" s="1">
         <f>Puskesmas!G15</f>
-        <v>86299.621799999994</v>
+        <v>114568.512275</v>
       </c>
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C16" s="1">
-        <v>-1.423</v>
+        <v>1.6144000000000001</v>
       </c>
       <c r="D16" s="1">
-        <v>17.143999999999998</v>
+        <v>19.0943</v>
       </c>
       <c r="E16" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F16" s="1">
         <f>Puskesmas!G16</f>
-        <v>114568.512275</v>
+        <v>98088.06147500001</v>
       </c>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C17" s="1">
-        <v>1.5449999999999999</v>
+        <v>-0.20682</v>
       </c>
       <c r="D17" s="1">
-        <v>19.071999999999999</v>
+        <v>20.052119999999999</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F17" s="1">
         <f>Puskesmas!G17</f>
-        <v>98088.06147500001</v>
+        <v>65146.784099999997</v>
       </c>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C18" s="1">
-        <v>5.2999999999999999E-2</v>
+        <v>-0.82450000000000001</v>
       </c>
       <c r="D18" s="1">
-        <v>20.032</v>
+        <v>18.1294</v>
       </c>
       <c r="E18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F18" s="1">
         <f>Puskesmas!G18</f>
-        <v>65146.784099999997</v>
+        <v>52558.355675000006</v>
       </c>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C19" s="1">
-        <v>-1.0740000000000001</v>
+        <v>5.4399999999999997E-2</v>
       </c>
       <c r="D19" s="1">
-        <v>17.899999999999999</v>
+        <v>18.332799999999999</v>
       </c>
       <c r="E19" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F19" s="1">
         <f>Puskesmas!G19</f>
-        <v>52558.355675000006</v>
+        <v>119644.90854999999</v>
       </c>
       <c r="G19" s="1"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="1">
-        <v>5.3999999999999999E-2</v>
-      </c>
-      <c r="D20" s="1">
-        <v>18.231000000000002</v>
-      </c>
-      <c r="E20" t="s">
-        <v>31</v>
-      </c>
-      <c r="F20" s="1">
-        <f>Puskesmas!G20</f>
-        <v>119644.90854999999</v>
-      </c>
-      <c r="G20" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1618,7 +1590,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{098AA237-CD4F-4868-9842-2B0C8D95453B}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
@@ -1655,16 +1627,16 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1">
-        <v>0.22</v>
+        <v>4.5199999999999997E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>18.391999999999999</v>
+        <v>18.264500000000002</v>
       </c>
       <c r="E2" t="str">
-        <f t="shared" ref="E2:E6" si="0">_xlfn.CONCAT("HZ",A2)</f>
+        <f t="shared" ref="E2:E5" si="0">_xlfn.CONCAT("HZ",A2)</f>
         <v>HZMbandaka</v>
       </c>
       <c r="F2" s="1">
@@ -1679,13 +1651,13 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1">
-        <v>0.92100000000000004</v>
+        <v>1.2185999999999999</v>
       </c>
       <c r="D3" s="1">
-        <v>19.881</v>
+        <v>19.7912</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" si="0"/>
@@ -1703,13 +1675,13 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1">
-        <v>-0.46600000000000003</v>
+        <v>-0.72570000000000001</v>
       </c>
       <c r="D4" s="1">
-        <v>18.231999999999999</v>
+        <v>18.124600000000001</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
@@ -1724,385 +1696,361 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C5" s="1">
-        <v>-0.20300000000000001</v>
+        <v>1.8699999999999999E-3</v>
       </c>
       <c r="D5" s="1">
-        <v>18.038</v>
+        <v>18.210999999999999</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
-        <v>HZBolenge_s</v>
+        <v>HZBolenge</v>
       </c>
       <c r="F5" s="1">
-        <v>3775.1895250000002</v>
+        <v>68536.694224999999</v>
       </c>
       <c r="G5" s="1">
-        <v>3775.1895250000002</v>
+        <v>133298.198925</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" s="1">
-        <v>-0.11700000000000001</v>
+        <v>0.35349999999999998</v>
       </c>
       <c r="D6" s="1">
-        <v>18.297000000000001</v>
+        <v>19.222999999999999</v>
       </c>
       <c r="E6" t="str">
-        <f t="shared" si="0"/>
-        <v>HZBolenge_l</v>
+        <f>_xlfn.CONCAT("HZ",A6)</f>
+        <v>HZBolomba</v>
       </c>
       <c r="F6" s="1">
-        <v>64761.504700000005</v>
+        <v>221127.34227500003</v>
       </c>
       <c r="G6" s="1">
-        <v>64761.504700000005</v>
+        <v>221127.34227500003</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C7" s="1">
-        <v>0.35099999999999998</v>
+        <v>1.38</v>
       </c>
       <c r="D7" s="1">
-        <v>19.091000000000001</v>
+        <v>18.3506</v>
       </c>
       <c r="E7" t="str">
-        <f>_xlfn.CONCAT("HZ",A7)</f>
-        <v>HZBolomba</v>
+        <f t="shared" ref="E7:E19" si="1">_xlfn.CONCAT("HZ",A7)</f>
+        <v>HZBomongo</v>
       </c>
       <c r="F7" s="1">
-        <v>221127.34227500003</v>
+        <v>88107.397450000004</v>
       </c>
       <c r="G7" s="1">
-        <v>221127.34227500003</v>
+        <v>88107.397450000004</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C8" s="1">
-        <v>1.5149999999999999</v>
+        <v>1.3486</v>
       </c>
       <c r="D8" s="1">
-        <v>18.442</v>
+        <v>20.382899999999999</v>
       </c>
       <c r="E8" t="str">
-        <f t="shared" ref="E8:E20" si="1">_xlfn.CONCAT("HZ",A8)</f>
-        <v>HZBomongo</v>
+        <f t="shared" si="1"/>
+        <v>HZDjombo</v>
       </c>
       <c r="F8" s="1">
-        <v>88107.397450000004</v>
+        <v>92383.804974999992</v>
       </c>
       <c r="G8" s="1">
-        <v>88107.397450000004</v>
+        <v>92383.804974999992</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C9" s="1">
-        <v>1.369</v>
+        <v>-1.1132</v>
       </c>
       <c r="D9" s="1">
-        <v>20.341000000000001</v>
+        <v>18.5334</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="1"/>
-        <v>HZDjombo</v>
+        <v>HZIboko</v>
       </c>
       <c r="F9" s="1">
-        <v>92383.804974999992</v>
+        <v>82515.513500000001</v>
       </c>
       <c r="G9" s="1">
-        <v>92383.804974999992</v>
+        <v>82515.513500000001</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C10" s="1">
-        <v>-0.94799999999999995</v>
+        <v>-0.30859999999999999</v>
       </c>
       <c r="D10" s="1">
-        <v>18.606000000000002</v>
+        <v>18.965199999999999</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="1"/>
-        <v>HZIboko</v>
+        <v>HZIngende</v>
       </c>
       <c r="F10" s="1">
-        <v>82515.513500000001</v>
+        <v>121623.91665000003</v>
       </c>
       <c r="G10" s="1">
-        <v>82515.513500000001</v>
+        <v>121623.91665000003</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C11" s="1">
-        <v>-0.44900000000000001</v>
+        <v>-0.61309999999999998</v>
       </c>
       <c r="D11" s="1">
-        <v>18.832999999999998</v>
+        <v>17.740200000000002</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="1"/>
-        <v>HZIngende</v>
+        <v>HZIrebu</v>
       </c>
       <c r="F11" s="1">
-        <v>121623.91665000003</v>
+        <v>29051.932274999999</v>
       </c>
       <c r="G11" s="1">
-        <v>121623.91665000003</v>
+        <v>29051.932274999999</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C12" s="1">
-        <v>-0.74399999999999999</v>
+        <v>-0.44059999999999999</v>
       </c>
       <c r="D12" s="1">
-        <v>17.663</v>
+        <v>17.7424</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="1"/>
-        <v>HZIrebu</v>
+        <v>HZLilanga Bobangi</v>
       </c>
       <c r="F12" s="1">
-        <v>29051.932274999999</v>
+        <v>66117.112875000006</v>
       </c>
       <c r="G12" s="1">
-        <v>29051.932274999999</v>
+        <v>66117.112875000006</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C13" s="1">
-        <v>0.18</v>
+        <v>0.86180000000000001</v>
       </c>
       <c r="D13" s="1">
-        <v>17.978000000000002</v>
+        <v>18.6755</v>
       </c>
       <c r="E13" t="str">
         <f t="shared" si="1"/>
-        <v>HZLilanga Bobangi</v>
+        <v>HZLolanga Mampoko</v>
       </c>
       <c r="F13" s="1">
-        <v>66117.112875000006</v>
+        <v>73921.670624999999</v>
       </c>
       <c r="G13" s="1">
-        <v>66117.112875000006</v>
+        <v>73921.670624999999</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C14" s="1">
-        <v>0.86499999999999999</v>
+        <v>-0.52459999999999996</v>
       </c>
       <c r="D14" s="1">
-        <v>18.713000000000001</v>
+        <v>19.425599999999999</v>
       </c>
       <c r="E14" t="str">
         <f t="shared" si="1"/>
-        <v>HZLolanga Mampoko</v>
+        <v>HZLotumbe</v>
       </c>
       <c r="F14" s="1">
-        <v>73921.670624999999</v>
+        <v>86299.621799999994</v>
       </c>
       <c r="G14" s="1">
-        <v>73921.670624999999</v>
+        <v>86299.621799999994</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C15" s="1">
-        <v>-0.68200000000000005</v>
+        <v>-1.0618000000000001</v>
       </c>
       <c r="D15" s="1">
-        <v>19.683</v>
+        <v>17.177399999999999</v>
       </c>
       <c r="E15" t="str">
         <f t="shared" si="1"/>
-        <v>HZLotumbe</v>
+        <v>HZLukolela</v>
       </c>
       <c r="F15" s="1">
-        <v>86299.621799999994</v>
+        <v>114568.512275</v>
       </c>
       <c r="G15" s="1">
-        <v>86299.621799999994</v>
+        <v>114568.512275</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C16" s="1">
-        <v>-1.423</v>
+        <v>1.6144000000000001</v>
       </c>
       <c r="D16" s="1">
-        <v>17.143999999999998</v>
+        <v>19.0943</v>
       </c>
       <c r="E16" t="str">
         <f t="shared" si="1"/>
-        <v>HZLukolela</v>
+        <v>HZMakanza</v>
       </c>
       <c r="F16" s="1">
-        <v>114568.512275</v>
+        <v>98088.06147500001</v>
       </c>
       <c r="G16" s="1">
-        <v>114568.512275</v>
+        <v>98088.06147500001</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C17" s="1">
-        <v>1.5449999999999999</v>
+        <v>-0.20682</v>
       </c>
       <c r="D17" s="1">
-        <v>19.071999999999999</v>
+        <v>20.052119999999999</v>
       </c>
       <c r="E17" t="str">
         <f t="shared" si="1"/>
-        <v>HZMakanza</v>
+        <v>HZMonieka</v>
       </c>
       <c r="F17" s="1">
-        <v>98088.06147500001</v>
+        <v>65146.784099999997</v>
       </c>
       <c r="G17" s="1">
-        <v>98088.06147500001</v>
+        <v>65146.784099999997</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C18" s="1">
-        <v>5.2999999999999999E-2</v>
+        <v>-0.82450000000000001</v>
       </c>
       <c r="D18" s="1">
-        <v>20.032</v>
+        <v>18.1294</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" si="1"/>
-        <v>HZMonieka</v>
+        <v>HZNtondo</v>
       </c>
       <c r="F18" s="1">
-        <v>65146.784099999997</v>
+        <v>52558.355675000006</v>
       </c>
       <c r="G18" s="1">
-        <v>65146.784099999997</v>
+        <v>52558.355675000006</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
         <v>27</v>
       </c>
-      <c r="B19" t="s">
-        <v>29</v>
-      </c>
       <c r="C19" s="1">
-        <v>-1.0740000000000001</v>
+        <v>5.4399999999999997E-2</v>
       </c>
       <c r="D19" s="1">
-        <v>17.899999999999999</v>
+        <v>18.332799999999999</v>
       </c>
       <c r="E19" t="str">
         <f t="shared" si="1"/>
-        <v>HZNtondo</v>
+        <v>HZWangata</v>
       </c>
       <c r="F19" s="1">
-        <v>52558.355675000006</v>
+        <v>119644.90854999999</v>
       </c>
       <c r="G19" s="1">
-        <v>52558.355675000006</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="1">
-        <v>5.3999999999999999E-2</v>
-      </c>
-      <c r="D20" s="1">
-        <v>18.231000000000002</v>
-      </c>
-      <c r="E20" t="str">
-        <f t="shared" si="1"/>
-        <v>HZWangata</v>
-      </c>
-      <c r="F20" s="1">
-        <v>119644.90854999999</v>
-      </c>
-      <c r="G20" s="1">
         <v>119644.90854999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modify the health area coordinates
The current version has a reduced set of health areas for one province based on K-means clustering
</commit_message>
<xml_diff>
--- a/Data/national-puskesmas-VSC.xlsx
+++ b/Data/national-puskesmas-VSC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fc1fb\Models\Vax SC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97917454-86B0-44A7-B611-6211CBC78A71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31833055-3BAB-4AD3-ACC3-932F50C856F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="3" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="71">
   <si>
     <t>Name</t>
   </si>
@@ -68,57 +68,12 @@
     <t>Initial Demand</t>
   </si>
   <si>
-    <t>Mbandaka</t>
-  </si>
-  <si>
-    <t>Basankusu</t>
-  </si>
-  <si>
-    <t>Bikoro</t>
-  </si>
-  <si>
-    <t>Bolomba</t>
-  </si>
-  <si>
-    <t>Bomongo</t>
-  </si>
-  <si>
-    <t>Djombo</t>
-  </si>
-  <si>
-    <t>Iboko</t>
-  </si>
-  <si>
-    <t>Ingende</t>
-  </si>
-  <si>
-    <t>Irebu</t>
-  </si>
-  <si>
-    <t>Lilanga Bobangi</t>
-  </si>
-  <si>
-    <t>Lolanga Mampoko</t>
-  </si>
-  <si>
     <t>Lotumbe</t>
   </si>
   <si>
-    <t>Lukolela</t>
-  </si>
-  <si>
-    <t>Makanza</t>
-  </si>
-  <si>
-    <t>Monieka</t>
-  </si>
-  <si>
     <t>Ntondo</t>
   </si>
   <si>
-    <t>Wangata</t>
-  </si>
-  <si>
     <t>Equateur</t>
   </si>
   <si>
@@ -186,6 +141,114 @@
   </si>
   <si>
     <t>Bolenge</t>
+  </si>
+  <si>
+    <t>Bokeka</t>
+  </si>
+  <si>
+    <t>Bosongo</t>
+  </si>
+  <si>
+    <t>Botunu</t>
+  </si>
+  <si>
+    <t>De la Rive</t>
+  </si>
+  <si>
+    <t>Djoa</t>
+  </si>
+  <si>
+    <t>Itumba</t>
+  </si>
+  <si>
+    <t>Iyembe Monene</t>
+  </si>
+  <si>
+    <t>Losako</t>
+  </si>
+  <si>
+    <t>Maanga</t>
+  </si>
+  <si>
+    <t>Mampoko</t>
+  </si>
+  <si>
+    <t>Nkondi</t>
+  </si>
+  <si>
+    <t>Penzele</t>
+  </si>
+  <si>
+    <t>Bafumba</t>
+  </si>
+  <si>
+    <t>Batsina Lifumba</t>
+  </si>
+  <si>
+    <t>Bobanga</t>
+  </si>
+  <si>
+    <t>Bolombo</t>
+  </si>
+  <si>
+    <t>Bongila</t>
+  </si>
+  <si>
+    <t>Bonsole Lofosola</t>
+  </si>
+  <si>
+    <t>Bosoisongo</t>
+  </si>
+  <si>
+    <t>Boyeka</t>
+  </si>
+  <si>
+    <t>Buburu</t>
+  </si>
+  <si>
+    <t>Ikoko Motaka</t>
+  </si>
+  <si>
+    <t>Ilambasa</t>
+  </si>
+  <si>
+    <t>Libanda</t>
+  </si>
+  <si>
+    <t>Ligbalo</t>
+  </si>
+  <si>
+    <t>Likuba</t>
+  </si>
+  <si>
+    <t>Lobengo</t>
+  </si>
+  <si>
+    <t>Lobuya</t>
+  </si>
+  <si>
+    <t>Lokolo Moko</t>
+  </si>
+  <si>
+    <t>Lokongo</t>
+  </si>
+  <si>
+    <t>Makako</t>
+  </si>
+  <si>
+    <t>Mambenga 1</t>
+  </si>
+  <si>
+    <t>Monzambi</t>
+  </si>
+  <si>
+    <t>Salongo</t>
+  </si>
+  <si>
+    <t>Waka</t>
+  </si>
+  <si>
+    <t>Boso-Mbuki</t>
   </si>
 </sst>
 </file>
@@ -1079,7 +1142,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1092,7 +1155,7 @@
       </c>
       <c r="E2">
         <f>SUM(ProvincialPublicHealth!F2:F4)</f>
-        <v>1889761.5028750007</v>
+        <v>1824999.9981750008</v>
       </c>
     </row>
   </sheetData>
@@ -1132,7 +1195,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -1144,11 +1207,11 @@
         <v>18.264500000000002</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F2">
         <f>SUM(DistrictHealthOffice!F2:F19)</f>
-        <v>1889761.5028750007</v>
+        <v>1824999.9981750008</v>
       </c>
     </row>
   </sheetData>
@@ -1189,10 +1252,10 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1">
         <v>4.5199999999999997E-2</v>
@@ -1201,20 +1264,20 @@
         <v>18.264500000000002</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F2" s="1">
-        <f>Puskesmas!G2</f>
+        <f>SUM(Puskesmas!G2:G3)</f>
         <v>116041.84390000002</v>
       </c>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1">
         <v>1.2185999999999999</v>
@@ -1223,20 +1286,20 @@
         <v>19.7912</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F3" s="1">
-        <f>Puskesmas!G3</f>
+        <f>SUM(Puskesmas!G4:G6)</f>
         <v>206265.59529999999</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1">
         <v>-0.72570000000000001</v>
@@ -1245,20 +1308,20 @@
         <v>18.124600000000001</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F4" s="1">
-        <f>Puskesmas!G4</f>
+        <f>SUM(Puskesmas!G7:G9)</f>
         <v>123000.93025</v>
       </c>
       <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1">
         <v>1.8699999999999999E-3</v>
@@ -1267,20 +1330,20 @@
         <v>18.210999999999999</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F5" s="1">
-        <f>Puskesmas!G5</f>
-        <v>133298.198925</v>
+        <f>SUM(Puskesmas!G10:G11)</f>
+        <v>68536.694224999999</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1">
         <v>0.35349999999999998</v>
@@ -1289,20 +1352,20 @@
         <v>19.222999999999999</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F6" s="1">
-        <f>Puskesmas!G6</f>
-        <v>221127.34227500003</v>
+        <f>SUM(Puskesmas!G12:G16)</f>
+        <v>221127.34227500006</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C7" s="1">
         <v>1.38</v>
@@ -1311,20 +1374,20 @@
         <v>18.3506</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F7" s="1">
-        <f>Puskesmas!G7</f>
+        <f>SUM(Puskesmas!G17:G18)</f>
         <v>88107.397450000004</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C8" s="1">
         <v>1.3486</v>
@@ -1333,20 +1396,20 @@
         <v>20.382899999999999</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F8" s="1">
-        <f>Puskesmas!G8</f>
+        <f>SUM(Puskesmas!G19)</f>
         <v>92383.804974999992</v>
       </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1">
         <v>-1.1132</v>
@@ -1355,20 +1418,20 @@
         <v>18.5334</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F9" s="1">
-        <f>Puskesmas!G9</f>
+        <f>SUM(Puskesmas!G20)</f>
         <v>82515.513500000001</v>
       </c>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C10" s="1">
         <v>-0.30859999999999999</v>
@@ -1377,20 +1440,20 @@
         <v>18.965199999999999</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F10" s="1">
-        <f>Puskesmas!G10</f>
+        <f>SUM(Puskesmas!G21:G22)</f>
         <v>121623.91665000003</v>
       </c>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C11" s="1">
         <v>-0.61309999999999998</v>
@@ -1399,20 +1462,20 @@
         <v>17.740200000000002</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F11" s="1">
-        <f>Puskesmas!G11</f>
+        <f>SUM(Puskesmas!G23:G24)</f>
         <v>29051.932274999999</v>
       </c>
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C12" s="1">
         <v>-0.44059999999999999</v>
@@ -1421,20 +1484,20 @@
         <v>17.7424</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F12" s="1">
-        <f>Puskesmas!G12</f>
+        <f>SUM(Puskesmas!G25:G28)</f>
         <v>66117.112875000006</v>
       </c>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C13" s="1">
         <v>0.86180000000000001</v>
@@ -1443,20 +1506,20 @@
         <v>18.6755</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F13" s="1">
-        <f>Puskesmas!G13</f>
+        <f>SUM(Puskesmas!G29:G30)</f>
         <v>73921.670624999999</v>
       </c>
       <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C14" s="1">
         <v>-0.52459999999999996</v>
@@ -1465,20 +1528,20 @@
         <v>19.425599999999999</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F14" s="1">
-        <f>Puskesmas!G14</f>
+        <f>SUM(Puskesmas!G31:G32)</f>
         <v>86299.621799999994</v>
       </c>
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C15" s="1">
         <v>-1.0618000000000001</v>
@@ -1487,20 +1550,20 @@
         <v>17.177399999999999</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F15" s="1">
-        <f>Puskesmas!G15</f>
+        <f>SUM(Puskesmas!G33:G34)</f>
         <v>114568.512275</v>
       </c>
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C16" s="1">
         <v>1.6144000000000001</v>
@@ -1509,20 +1572,20 @@
         <v>19.0943</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F16" s="1">
-        <f>Puskesmas!G16</f>
+        <f>SUM(Puskesmas!G35:G38)</f>
         <v>98088.06147500001</v>
       </c>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C17" s="1">
         <v>-0.20682</v>
@@ -1531,20 +1594,20 @@
         <v>20.052119999999999</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F17" s="1">
-        <f>Puskesmas!G17</f>
+        <f>SUM(Puskesmas!G39)</f>
         <v>65146.784099999997</v>
       </c>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C18" s="1">
         <v>-0.82450000000000001</v>
@@ -1553,20 +1616,20 @@
         <v>18.1294</v>
       </c>
       <c r="E18" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F18" s="1">
-        <f>Puskesmas!G18</f>
+        <f>SUM(Puskesmas!G40)</f>
         <v>52558.355675000006</v>
       </c>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C19" s="1">
         <v>5.4399999999999997E-2</v>
@@ -1575,10 +1638,10 @@
         <v>18.332799999999999</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F19" s="1">
-        <f>Puskesmas!G19</f>
+        <f>SUM(Puskesmas!G41)</f>
         <v>119644.90854999999</v>
       </c>
       <c r="G19" s="1"/>
@@ -1590,7 +1653,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{098AA237-CD4F-4868-9842-2B0C8D95453B}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
@@ -1623,434 +1686,922 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>10</v>
+      <c r="A2" t="s">
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="1">
-        <v>4.5199999999999997E-2</v>
-      </c>
-      <c r="D2" s="1">
-        <v>18.264500000000002</v>
-      </c>
-      <c r="E2" t="str">
-        <f t="shared" ref="E2:E5" si="0">_xlfn.CONCAT("HZ",A2)</f>
-        <v>HZMbandaka</v>
+        <v>12</v>
+      </c>
+      <c r="C2">
+        <v>5.36622E-2</v>
+      </c>
+      <c r="D2">
+        <v>18.333210000000001</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
       </c>
       <c r="F2" s="1">
-        <v>116041.84390000002</v>
+        <v>58020.921950000011</v>
       </c>
       <c r="G2" s="1">
-        <v>116041.84390000002</v>
+        <v>58020.921950000011</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>11</v>
+      <c r="A3" t="s">
+        <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1.2185999999999999</v>
-      </c>
-      <c r="D3" s="1">
-        <v>19.7912</v>
-      </c>
-      <c r="E3" t="str">
-        <f t="shared" si="0"/>
-        <v>HZBasankusu</v>
+        <v>12</v>
+      </c>
+      <c r="C3">
+        <v>5.475E-2</v>
+      </c>
+      <c r="D3">
+        <v>18.266449999999999</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
       </c>
       <c r="F3" s="1">
-        <v>206265.59529999999</v>
+        <v>58020.921950000011</v>
       </c>
       <c r="G3" s="1">
-        <v>206265.59529999999</v>
+        <v>58020.921950000011</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1">
-        <v>-0.72570000000000001</v>
+        <v>0.69919830000000005</v>
       </c>
       <c r="D4" s="1">
-        <v>18.124600000000001</v>
-      </c>
-      <c r="E4" t="str">
-        <f t="shared" si="0"/>
-        <v>HZBikoro</v>
+        <v>19.987680000000001</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
       </c>
       <c r="F4" s="1">
-        <v>123000.93025</v>
+        <v>68755.198433333324</v>
       </c>
       <c r="G4" s="1">
-        <v>123000.93025</v>
+        <v>68755.198433333324</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C5" s="1">
-        <v>1.8699999999999999E-3</v>
+        <v>1.2224767000000001</v>
       </c>
       <c r="D5" s="1">
-        <v>18.210999999999999</v>
-      </c>
-      <c r="E5" t="str">
-        <f t="shared" si="0"/>
-        <v>HZBolenge</v>
+        <v>19.789449999999999</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
       </c>
       <c r="F5" s="1">
-        <v>68536.694224999999</v>
+        <v>68755.198433333324</v>
       </c>
       <c r="G5" s="1">
-        <v>133298.198925</v>
+        <v>68755.198433333324</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C6" s="1">
-        <v>0.35349999999999998</v>
+        <v>1.0065583</v>
       </c>
       <c r="D6" s="1">
-        <v>19.222999999999999</v>
-      </c>
-      <c r="E6" t="str">
-        <f>_xlfn.CONCAT("HZ",A6)</f>
-        <v>HZBolomba</v>
+        <v>20.192969999999999</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
       </c>
       <c r="F6" s="1">
-        <v>221127.34227500003</v>
+        <v>68755.198433333324</v>
       </c>
       <c r="G6" s="1">
-        <v>221127.34227500003</v>
+        <v>68755.198433333324</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C7" s="1">
-        <v>1.38</v>
+        <v>-0.69606670000000004</v>
       </c>
       <c r="D7" s="1">
-        <v>18.3506</v>
-      </c>
-      <c r="E7" t="str">
-        <f t="shared" ref="E7:E19" si="1">_xlfn.CONCAT("HZ",A7)</f>
-        <v>HZBomongo</v>
+        <v>18.267555000000002</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
       </c>
       <c r="F7" s="1">
-        <v>88107.397450000004</v>
+        <v>41000.310083333337</v>
       </c>
       <c r="G7" s="1">
-        <v>88107.397450000004</v>
+        <v>41000.310083333337</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C8" s="1">
-        <v>1.3486</v>
+        <v>-0.71287670000000003</v>
       </c>
       <c r="D8" s="1">
-        <v>20.382899999999999</v>
-      </c>
-      <c r="E8" t="str">
-        <f t="shared" si="1"/>
-        <v>HZDjombo</v>
+        <v>17.865138300000002</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
       </c>
       <c r="F8" s="1">
-        <v>92383.804974999992</v>
+        <v>41000.310083333337</v>
       </c>
       <c r="G8" s="1">
-        <v>92383.804974999992</v>
+        <v>41000.310083333337</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C9" s="1">
-        <v>-1.1132</v>
+        <v>-0.28829830000000001</v>
       </c>
       <c r="D9" s="1">
-        <v>18.5334</v>
-      </c>
-      <c r="E9" t="str">
-        <f t="shared" si="1"/>
-        <v>HZIboko</v>
+        <v>18.2235683</v>
+      </c>
+      <c r="E9" t="s">
+        <v>18</v>
       </c>
       <c r="F9" s="1">
-        <v>82515.513500000001</v>
+        <v>41000.310083333337</v>
       </c>
       <c r="G9" s="1">
-        <v>82515.513500000001</v>
+        <v>41000.310083333337</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C10" s="1">
-        <v>-0.30859999999999999</v>
+        <v>-6.1499999999999999E-4</v>
       </c>
       <c r="D10" s="1">
-        <v>18.965199999999999</v>
-      </c>
-      <c r="E10" t="str">
-        <f t="shared" si="1"/>
-        <v>HZIngende</v>
+        <v>18.217569999999998</v>
+      </c>
+      <c r="E10" t="s">
+        <v>33</v>
       </c>
       <c r="F10" s="1">
-        <v>121623.91665000003</v>
+        <v>34268.3471125</v>
       </c>
       <c r="G10" s="1">
-        <v>121623.91665000003</v>
+        <v>34268.3471125</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C11" s="1">
-        <v>-0.61309999999999998</v>
+        <v>-0.132994</v>
       </c>
       <c r="D11" s="1">
-        <v>17.740200000000002</v>
-      </c>
-      <c r="E11" t="str">
-        <f t="shared" si="1"/>
-        <v>HZIrebu</v>
+        <v>18.278957699999999</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
       </c>
       <c r="F11" s="1">
-        <v>29051.932274999999</v>
+        <v>34268.3471125</v>
       </c>
       <c r="G11" s="1">
-        <v>29051.932274999999</v>
+        <v>34268.3471125</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="1">
+        <v>3.5286699999999997E-2</v>
+      </c>
+      <c r="D12" s="1">
+        <v>19.286788300000001</v>
+      </c>
+      <c r="E12" t="s">
         <v>19</v>
       </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="1">
-        <v>-0.44059999999999999</v>
-      </c>
-      <c r="D12" s="1">
-        <v>17.7424</v>
-      </c>
-      <c r="E12" t="str">
-        <f t="shared" si="1"/>
-        <v>HZLilanga Bobangi</v>
-      </c>
       <c r="F12" s="1">
-        <v>66117.112875000006</v>
+        <v>44225.468455000009</v>
       </c>
       <c r="G12" s="1">
-        <v>66117.112875000006</v>
+        <v>44225.468455000009</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1">
-        <v>0.86180000000000001</v>
+        <v>7.2531700000000005E-2</v>
       </c>
       <c r="D13" s="1">
-        <v>18.6755</v>
-      </c>
-      <c r="E13" t="str">
-        <f t="shared" si="1"/>
-        <v>HZLolanga Mampoko</v>
+        <v>18.843871700000001</v>
+      </c>
+      <c r="E13" t="s">
+        <v>19</v>
       </c>
       <c r="F13" s="1">
-        <v>73921.670624999999</v>
+        <v>44225.468455000009</v>
       </c>
       <c r="G13" s="1">
-        <v>73921.670624999999</v>
+        <v>44225.468455000009</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C14" s="1">
-        <v>-0.52459999999999996</v>
+        <v>0.48443000000000003</v>
       </c>
       <c r="D14" s="1">
-        <v>19.425599999999999</v>
-      </c>
-      <c r="E14" t="str">
-        <f t="shared" si="1"/>
-        <v>HZLotumbe</v>
+        <v>19.246960000000001</v>
+      </c>
+      <c r="E14" t="s">
+        <v>19</v>
       </c>
       <c r="F14" s="1">
-        <v>86299.621799999994</v>
+        <v>44225.468455000009</v>
       </c>
       <c r="G14" s="1">
-        <v>86299.621799999994</v>
+        <v>44225.468455000009</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C15" s="1">
-        <v>-1.0618000000000001</v>
+        <v>1.054095</v>
       </c>
       <c r="D15" s="1">
-        <v>17.177399999999999</v>
-      </c>
-      <c r="E15" t="str">
-        <f t="shared" si="1"/>
-        <v>HZLukolela</v>
+        <v>19.290103299999998</v>
+      </c>
+      <c r="E15" t="s">
+        <v>19</v>
       </c>
       <c r="F15" s="1">
-        <v>114568.512275</v>
+        <v>44225.468455000009</v>
       </c>
       <c r="G15" s="1">
-        <v>114568.512275</v>
+        <v>44225.468455000009</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C16" s="1">
-        <v>1.6144000000000001</v>
+        <v>0.30522329999999998</v>
       </c>
       <c r="D16" s="1">
-        <v>19.0943</v>
-      </c>
-      <c r="E16" t="str">
-        <f t="shared" si="1"/>
-        <v>HZMakanza</v>
+        <v>18.536603299999999</v>
+      </c>
+      <c r="E16" t="s">
+        <v>19</v>
       </c>
       <c r="F16" s="1">
-        <v>98088.06147500001</v>
+        <v>44225.468455000009</v>
       </c>
       <c r="G16" s="1">
-        <v>98088.06147500001</v>
+        <v>44225.468455000009</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C17" s="1">
-        <v>-0.20682</v>
+        <v>1.4394283329999999</v>
       </c>
       <c r="D17" s="1">
-        <v>20.052119999999999</v>
-      </c>
-      <c r="E17" t="str">
-        <f t="shared" si="1"/>
-        <v>HZMonieka</v>
+        <v>18.038969999999999</v>
+      </c>
+      <c r="E17" t="s">
+        <v>20</v>
       </c>
       <c r="F17" s="1">
-        <v>65146.784099999997</v>
+        <v>44053.698725000002</v>
       </c>
       <c r="G17" s="1">
-        <v>65146.784099999997</v>
+        <v>44053.698725000002</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C18" s="1">
-        <v>-0.82450000000000001</v>
+        <v>1.4506867000000001</v>
       </c>
       <c r="D18" s="1">
-        <v>18.1294</v>
-      </c>
-      <c r="E18" t="str">
-        <f t="shared" si="1"/>
-        <v>HZNtondo</v>
+        <v>18.393948300000002</v>
+      </c>
+      <c r="E18" t="s">
+        <v>20</v>
       </c>
       <c r="F18" s="1">
-        <v>52558.355675000006</v>
+        <v>44053.698725000002</v>
       </c>
       <c r="G18" s="1">
-        <v>52558.355675000006</v>
+        <v>44053.698725000002</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1.429296667</v>
+      </c>
+      <c r="D19" s="1">
+        <v>20.462073332999999</v>
+      </c>
+      <c r="E19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="1">
+        <v>92383.804974999992</v>
+      </c>
+      <c r="G19" s="1">
+        <v>92383.804974999992</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="1">
+        <v>-0.92937999999999998</v>
+      </c>
+      <c r="D20" s="1">
+        <v>18.616076700000001</v>
+      </c>
+      <c r="E20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20" s="1">
+        <v>82515.513500000001</v>
+      </c>
+      <c r="G20" s="1">
+        <v>82515.513500000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="1">
+        <v>-0.52747500000000003</v>
+      </c>
+      <c r="D21" s="1">
+        <v>18.6058983</v>
+      </c>
+      <c r="E21" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="1">
+        <v>60811.958325000014</v>
+      </c>
+      <c r="G21" s="1">
+        <v>60811.958325000014</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22">
+        <v>-0.51719669999999995</v>
+      </c>
+      <c r="D22">
+        <v>18.993763300000001</v>
+      </c>
+      <c r="E22" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="1">
+        <v>60811.958325000014</v>
+      </c>
+      <c r="G22" s="1">
+        <v>60811.958325000014</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23">
+        <v>-0.64078829999999998</v>
+      </c>
+      <c r="D23">
+        <v>17.702921700000001</v>
+      </c>
+      <c r="E23" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" s="1">
+        <v>14525.9661375</v>
+      </c>
+      <c r="G23" s="1">
+        <v>14525.9661375</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24">
+        <v>-0.83704060000000002</v>
+      </c>
+      <c r="D24">
+        <v>17.510778500000001</v>
+      </c>
+      <c r="E24" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="1">
+        <v>14525.9661375</v>
+      </c>
+      <c r="G24" s="1">
+        <v>14525.9661375</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25">
+        <v>0.50983690000000004</v>
+      </c>
+      <c r="D25">
+        <v>18.291140299999999</v>
+      </c>
+      <c r="E25" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" s="1">
+        <v>16529.278218750002</v>
+      </c>
+      <c r="G25" s="1">
+        <v>16529.278218750002</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26">
+        <v>-8.2076800000000005E-2</v>
+      </c>
+      <c r="D26">
+        <v>18.089138699999999</v>
+      </c>
+      <c r="E26" t="s">
+        <v>25</v>
+      </c>
+      <c r="F26" s="1">
+        <v>16529.278218750002</v>
+      </c>
+      <c r="G26" s="1">
+        <v>16529.278218750002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27">
+        <v>0.77745819999999999</v>
+      </c>
+      <c r="D27">
+        <v>18.332442400000001</v>
+      </c>
+      <c r="E27" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" s="1">
+        <v>16529.278218750002</v>
+      </c>
+      <c r="G27" s="1">
+        <v>16529.278218750002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28">
+        <v>-0.27843449999999997</v>
+      </c>
+      <c r="D28">
+        <v>17.9063135</v>
+      </c>
+      <c r="E28" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" s="1">
+        <v>16529.278218750002</v>
+      </c>
+      <c r="G28" s="1">
+        <v>16529.278218750002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29">
+        <v>0.86187670000000005</v>
+      </c>
+      <c r="D29">
+        <v>18.674713300000001</v>
+      </c>
+      <c r="E29" t="s">
         <v>26</v>
       </c>
-      <c r="B19" t="s">
+      <c r="F29" s="1">
+        <v>36960.835312499999</v>
+      </c>
+      <c r="G29" s="1">
+        <v>36960.835312499999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30">
+        <v>0.83048330000000004</v>
+      </c>
+      <c r="D30">
+        <v>18.874023300000001</v>
+      </c>
+      <c r="E30" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="1">
+        <v>36960.835312499999</v>
+      </c>
+      <c r="G30" s="1">
+        <v>36960.835312499999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31">
+        <v>-0.92481780000000002</v>
+      </c>
+      <c r="D31">
+        <v>19.963625100000002</v>
+      </c>
+      <c r="E31" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="1">
-        <v>5.4399999999999997E-2</v>
-      </c>
-      <c r="D19" s="1">
-        <v>18.332799999999999</v>
-      </c>
-      <c r="E19" t="str">
-        <f t="shared" si="1"/>
-        <v>HZWangata</v>
-      </c>
-      <c r="F19" s="1">
+      <c r="F31" s="1">
+        <v>43149.810899999997</v>
+      </c>
+      <c r="G31" s="1">
+        <v>43149.810899999997</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32">
+        <v>-0.52240330000000001</v>
+      </c>
+      <c r="D32">
+        <v>19.4239067</v>
+      </c>
+      <c r="E32" t="s">
+        <v>27</v>
+      </c>
+      <c r="F32" s="1">
+        <v>43149.810899999997</v>
+      </c>
+      <c r="G32" s="1">
+        <v>43149.810899999997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33">
+        <v>-1.0625382999999999</v>
+      </c>
+      <c r="D33">
+        <v>17.167231699999999</v>
+      </c>
+      <c r="E33" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" s="1">
+        <v>57284.2561375</v>
+      </c>
+      <c r="G33" s="1">
+        <v>57284.2561375</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>45</v>
+      </c>
+      <c r="B34" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34">
+        <v>-1.6064000000000001</v>
+      </c>
+      <c r="D34">
+        <v>17.036096700000002</v>
+      </c>
+      <c r="E34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F34" s="1">
+        <v>57284.2561375</v>
+      </c>
+      <c r="G34" s="1">
+        <v>57284.2561375</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35">
+        <v>1.3631783</v>
+      </c>
+      <c r="D35">
+        <v>18.910348299999999</v>
+      </c>
+      <c r="E35" t="s">
+        <v>29</v>
+      </c>
+      <c r="F35" s="1">
+        <v>24522.015368750002</v>
+      </c>
+      <c r="G35" s="1">
+        <v>24522.015368750002</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36">
+        <v>1.61785</v>
+      </c>
+      <c r="D36">
+        <v>19.115331699999999</v>
+      </c>
+      <c r="E36" t="s">
+        <v>29</v>
+      </c>
+      <c r="F36" s="1">
+        <v>24522.015368750002</v>
+      </c>
+      <c r="G36" s="1">
+        <v>24522.015368750002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37">
+        <v>1.052738</v>
+      </c>
+      <c r="D37">
+        <v>18.450583900000002</v>
+      </c>
+      <c r="E37" t="s">
+        <v>29</v>
+      </c>
+      <c r="F37" s="1">
+        <v>24522.015368750002</v>
+      </c>
+      <c r="G37" s="1">
+        <v>24522.015368750002</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38">
+        <v>1.8413383000000001</v>
+      </c>
+      <c r="D38">
+        <v>19.562101699999999</v>
+      </c>
+      <c r="E38" t="s">
+        <v>29</v>
+      </c>
+      <c r="F38" s="1">
+        <v>24522.015368750002</v>
+      </c>
+      <c r="G38" s="1">
+        <v>24522.015368750002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39">
+        <v>0.1700538</v>
+      </c>
+      <c r="D39">
+        <v>19.9345809</v>
+      </c>
+      <c r="E39" t="s">
+        <v>30</v>
+      </c>
+      <c r="F39" s="1">
+        <v>65146.784099999997</v>
+      </c>
+      <c r="G39" s="1">
+        <v>65146.784099999997</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40">
+        <v>-0.97267999999999999</v>
+      </c>
+      <c r="D40">
+        <v>18.132546699999999</v>
+      </c>
+      <c r="E40" t="s">
+        <v>31</v>
+      </c>
+      <c r="F40" s="1">
+        <v>52558.355675000006</v>
+      </c>
+      <c r="G40" s="1">
+        <v>52558.355675000006</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>38</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41">
+        <v>4.1486599999999998E-2</v>
+      </c>
+      <c r="D41">
+        <v>18.239670499999999</v>
+      </c>
+      <c r="E41" t="s">
+        <v>32</v>
+      </c>
+      <c r="F41" s="1">
         <v>119644.90854999999</v>
       </c>
-      <c r="G19" s="1">
+      <c r="G41" s="1">
         <v>119644.90854999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modify pop centre code
Toward parameter variation tests, a new column was added to the database for adjustment factor which is multiplied to rollout speed (given by experiment) to create a new average demand based on rollout speed
</commit_message>
<xml_diff>
--- a/Data/national-puskesmas-VSC.xlsx
+++ b/Data/national-puskesmas-VSC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fc1fb\Models\Vax SC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31833055-3BAB-4AD3-ACC3-932F50C856F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6C7C43-EDA2-4623-83C4-BDA1E13FEFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15225" activeTab="3" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="14775" activeTab="2" xr2:uid="{FA23C16F-3C1C-4E68-AD36-4215747A6BE9}"/>
   </bookViews>
   <sheets>
     <sheet name="NationalOffice" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="72">
   <si>
     <t>Name</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t>Boso-Mbuki</t>
+  </si>
+  <si>
+    <t>Demand Factor</t>
   </si>
 </sst>
 </file>
@@ -1249,6 +1252,9 @@
       <c r="F1" t="s">
         <v>9</v>
       </c>
+      <c r="G1" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1270,7 +1276,10 @@
         <f>SUM(Puskesmas!G2:G3)</f>
         <v>116041.84390000002</v>
       </c>
-      <c r="G2" s="1"/>
+      <c r="G2" s="1">
+        <f>F2/SUM($F$2:$F$19)</f>
+        <v>6.358457206358456E-2</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1292,7 +1301,10 @@
         <f>SUM(Puskesmas!G4:G6)</f>
         <v>206265.59529999999</v>
       </c>
-      <c r="G3" s="1"/>
+      <c r="G3" s="1">
+        <f t="shared" ref="G3:G19" si="0">F3/SUM($F$2:$F$19)</f>
+        <v>0.11302224411302218</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -1314,7 +1326,10 @@
         <f>SUM(Puskesmas!G7:G9)</f>
         <v>123000.93025</v>
       </c>
-      <c r="G4" s="1"/>
+      <c r="G4" s="1">
+        <f t="shared" si="0"/>
+        <v>6.739777006739775E-2</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -1336,7 +1351,10 @@
         <f>SUM(Puskesmas!G10:G11)</f>
         <v>68536.694224999999</v>
       </c>
-      <c r="G5" s="1"/>
+      <c r="G5" s="1">
+        <f t="shared" si="0"/>
+        <v>3.7554353037554333E-2</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -1358,7 +1376,10 @@
         <f>SUM(Puskesmas!G12:G16)</f>
         <v>221127.34227500006</v>
       </c>
-      <c r="G6" s="1"/>
+      <c r="G6" s="1">
+        <f t="shared" si="0"/>
+        <v>0.12116566712116565</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -1380,7 +1401,10 @@
         <f>SUM(Puskesmas!G17:G18)</f>
         <v>88107.397450000004</v>
       </c>
-      <c r="G7" s="1"/>
+      <c r="G7" s="1">
+        <f t="shared" si="0"/>
+        <v>4.8278026048278008E-2</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -1402,7 +1426,10 @@
         <f>SUM(Puskesmas!G19)</f>
         <v>92383.804974999992</v>
       </c>
-      <c r="G8" s="1"/>
+      <c r="G8" s="1">
+        <f t="shared" si="0"/>
+        <v>5.0621263050621236E-2</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -1424,7 +1451,10 @@
         <f>SUM(Puskesmas!G20)</f>
         <v>82515.513500000001</v>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" s="1">
+        <f t="shared" si="0"/>
+        <v>4.5213980045213958E-2</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -1446,7 +1476,10 @@
         <f>SUM(Puskesmas!G21:G22)</f>
         <v>121623.91665000003</v>
       </c>
-      <c r="G10" s="1"/>
+      <c r="G10" s="1">
+        <f t="shared" si="0"/>
+        <v>6.6643242066643224E-2</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -1468,7 +1501,10 @@
         <f>SUM(Puskesmas!G23:G24)</f>
         <v>29051.932274999999</v>
       </c>
-      <c r="G11" s="1"/>
+      <c r="G11" s="1">
+        <f t="shared" si="0"/>
+        <v>1.591886701591886E-2</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -1490,7 +1526,10 @@
         <f>SUM(Puskesmas!G25:G28)</f>
         <v>66117.112875000006</v>
       </c>
-      <c r="G12" s="1"/>
+      <c r="G12" s="1">
+        <f t="shared" si="0"/>
+        <v>3.6228555036228544E-2</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -1512,7 +1551,10 @@
         <f>SUM(Puskesmas!G29:G30)</f>
         <v>73921.670624999999</v>
       </c>
-      <c r="G13" s="1"/>
+      <c r="G13" s="1">
+        <f t="shared" si="0"/>
+        <v>4.0505025040505009E-2</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -1534,7 +1576,10 @@
         <f>SUM(Puskesmas!G31:G32)</f>
         <v>86299.621799999994</v>
       </c>
-      <c r="G14" s="1"/>
+      <c r="G14" s="1">
+        <f t="shared" si="0"/>
+        <v>4.7287464047287439E-2</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -1556,7 +1601,10 @@
         <f>SUM(Puskesmas!G33:G34)</f>
         <v>114568.512275</v>
       </c>
-      <c r="G15" s="1"/>
+      <c r="G15" s="1">
+        <f t="shared" si="0"/>
+        <v>6.2777267062777239E-2</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -1578,7 +1626,10 @@
         <f>SUM(Puskesmas!G35:G38)</f>
         <v>98088.06147500001</v>
       </c>
-      <c r="G16" s="1"/>
+      <c r="G16" s="1">
+        <f t="shared" si="0"/>
+        <v>5.3746883053746863E-2</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
@@ -1600,7 +1651,10 @@
         <f>SUM(Puskesmas!G39)</f>
         <v>65146.784099999997</v>
       </c>
-      <c r="G17" s="1"/>
+      <c r="G17" s="1">
+        <f t="shared" si="0"/>
+        <v>3.5696868035696848E-2</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
@@ -1622,7 +1676,10 @@
         <f>SUM(Puskesmas!G40)</f>
         <v>52558.355675000006</v>
       </c>
-      <c r="G18" s="1"/>
+      <c r="G18" s="1">
+        <f t="shared" si="0"/>
+        <v>2.879909902879909E-2</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -1644,7 +1701,10 @@
         <f>SUM(Puskesmas!G41)</f>
         <v>119644.90854999999</v>
       </c>
-      <c r="G19" s="1"/>
+      <c r="G19" s="1">
+        <f t="shared" si="0"/>
+        <v>6.5558854065558822E-2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1653,7 +1713,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{098AA237-CD4F-4868-9842-2B0C8D95453B}">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" bestFit="1" customWidth="1"/>
@@ -1662,7 +1722,7 @@
     <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1684,8 +1744,11 @@
       <c r="G1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -1707,8 +1770,12 @@
       <c r="G2" s="1">
         <v>58020.921950000011</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2">
+        <f>F2/SUM($F$2:$F$41)</f>
+        <v>3.1792286031792301E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>66</v>
       </c>
@@ -1730,8 +1797,12 @@
       <c r="G3" s="1">
         <v>58020.921950000011</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3">
+        <f t="shared" ref="H3:H41" si="0">F3/SUM($F$2:$F$41)</f>
+        <v>3.1792286031792301E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -1753,8 +1824,12 @@
       <c r="G4" s="1">
         <v>68755.198433333324</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4">
+        <f t="shared" si="0"/>
+        <v>3.7674081371007417E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>47</v>
       </c>
@@ -1776,8 +1851,12 @@
       <c r="G5" s="1">
         <v>68755.198433333324</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5">
+        <f t="shared" si="0"/>
+        <v>3.7674081371007417E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>69</v>
       </c>
@@ -1799,8 +1878,12 @@
       <c r="G6" s="1">
         <v>68755.198433333324</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6">
+        <f t="shared" si="0"/>
+        <v>3.7674081371007417E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
@@ -1822,8 +1905,12 @@
       <c r="G7" s="1">
         <v>41000.310083333337</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>2.2465923355799264E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>43</v>
       </c>
@@ -1845,8 +1932,12 @@
       <c r="G8" s="1">
         <v>41000.310083333337</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8">
+        <f t="shared" si="0"/>
+        <v>2.2465923355799264E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>46</v>
       </c>
@@ -1868,8 +1959,12 @@
       <c r="G9" s="1">
         <v>41000.310083333337</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9">
+        <f t="shared" si="0"/>
+        <v>2.2465923355799264E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>34</v>
       </c>
@@ -1891,8 +1986,12 @@
       <c r="G10" s="1">
         <v>34268.3471125</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>1.8777176518777181E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>52</v>
       </c>
@@ -1914,8 +2013,12 @@
       <c r="G11" s="1">
         <v>34268.3471125</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>1.8777176518777181E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>39</v>
       </c>
@@ -1937,8 +2040,12 @@
       <c r="G12" s="1">
         <v>44225.468455000009</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H12">
+        <f t="shared" si="0"/>
+        <v>2.4233133424233142E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>34</v>
       </c>
@@ -1960,8 +2067,12 @@
       <c r="G13" s="1">
         <v>44225.468455000009</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H13">
+        <f t="shared" si="0"/>
+        <v>2.4233133424233142E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
@@ -1983,8 +2094,12 @@
       <c r="G14" s="1">
         <v>44225.468455000009</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H14">
+        <f t="shared" si="0"/>
+        <v>2.4233133424233142E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>59</v>
       </c>
@@ -2006,8 +2121,12 @@
       <c r="G15" s="1">
         <v>44225.468455000009</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H15">
+        <f t="shared" si="0"/>
+        <v>2.4233133424233142E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>67</v>
       </c>
@@ -2029,8 +2148,12 @@
       <c r="G16" s="1">
         <v>44225.468455000009</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16">
+        <f t="shared" si="0"/>
+        <v>2.4233133424233142E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>55</v>
       </c>
@@ -2052,8 +2175,12 @@
       <c r="G17" s="1">
         <v>44053.698725000002</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H17">
+        <f t="shared" si="0"/>
+        <v>2.4139013024139018E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>58</v>
       </c>
@@ -2075,8 +2202,12 @@
       <c r="G18" s="1">
         <v>44053.698725000002</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18">
+        <f t="shared" si="0"/>
+        <v>2.4139013024139018E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
@@ -2098,8 +2229,12 @@
       <c r="G19" s="1">
         <v>92383.804974999992</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19">
+        <f t="shared" si="0"/>
+        <v>5.0621263050621271E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>64</v>
       </c>
@@ -2121,8 +2256,12 @@
       <c r="G20" s="1">
         <v>82515.513500000001</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20">
+        <f t="shared" si="0"/>
+        <v>4.5213980045213993E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>48</v>
       </c>
@@ -2144,8 +2283,12 @@
       <c r="G21" s="1">
         <v>60811.958325000014</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H21">
+        <f t="shared" si="0"/>
+        <v>3.3321621033321633E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>65</v>
       </c>
@@ -2167,8 +2310,12 @@
       <c r="G22" s="1">
         <v>60811.958325000014</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H22">
+        <f t="shared" si="0"/>
+        <v>3.3321621033321633E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -2190,8 +2337,12 @@
       <c r="G23" s="1">
         <v>14525.9661375</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H23">
+        <f t="shared" si="0"/>
+        <v>7.9594335079594351E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -2213,8 +2364,12 @@
       <c r="G24" s="1">
         <v>14525.9661375</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H24">
+        <f t="shared" si="0"/>
+        <v>7.9594335079594351E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -2236,8 +2391,12 @@
       <c r="G25" s="1">
         <v>16529.278218750002</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H25">
+        <f t="shared" si="0"/>
+        <v>9.0571387590571411E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>57</v>
       </c>
@@ -2259,8 +2418,12 @@
       <c r="G26" s="1">
         <v>16529.278218750002</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H26">
+        <f t="shared" si="0"/>
+        <v>9.0571387590571411E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>63</v>
       </c>
@@ -2282,8 +2445,12 @@
       <c r="G27" s="1">
         <v>16529.278218750002</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H27">
+        <f t="shared" si="0"/>
+        <v>9.0571387590571411E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>68</v>
       </c>
@@ -2305,8 +2472,12 @@
       <c r="G28" s="1">
         <v>16529.278218750002</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H28">
+        <f t="shared" si="0"/>
+        <v>9.0571387590571411E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>44</v>
       </c>
@@ -2328,8 +2499,12 @@
       <c r="G29" s="1">
         <v>36960.835312499999</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H29">
+        <f t="shared" si="0"/>
+        <v>2.0252512520252515E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>70</v>
       </c>
@@ -2351,8 +2526,12 @@
       <c r="G30" s="1">
         <v>36960.835312499999</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H30">
+        <f t="shared" si="0"/>
+        <v>2.0252512520252515E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -2374,8 +2553,12 @@
       <c r="G31" s="1">
         <v>43149.810899999997</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H31">
+        <f t="shared" si="0"/>
+        <v>2.3643732023643737E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>10</v>
       </c>
@@ -2397,8 +2580,12 @@
       <c r="G32" s="1">
         <v>43149.810899999997</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H32">
+        <f t="shared" si="0"/>
+        <v>2.3643732023643737E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -2420,8 +2607,12 @@
       <c r="G33" s="1">
         <v>57284.2561375</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H33">
+        <f t="shared" si="0"/>
+        <v>3.1388633531388641E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>45</v>
       </c>
@@ -2443,8 +2634,12 @@
       <c r="G34" s="1">
         <v>57284.2561375</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H34">
+        <f t="shared" si="0"/>
+        <v>3.1388633531388641E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>50</v>
       </c>
@@ -2466,8 +2661,12 @@
       <c r="G35" s="1">
         <v>24522.015368750002</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H35">
+        <f t="shared" si="0"/>
+        <v>1.3436720763436725E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>60</v>
       </c>
@@ -2489,8 +2688,12 @@
       <c r="G36" s="1">
         <v>24522.015368750002</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H36">
+        <f t="shared" si="0"/>
+        <v>1.3436720763436725E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>61</v>
       </c>
@@ -2512,8 +2715,12 @@
       <c r="G37" s="1">
         <v>24522.015368750002</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H37">
+        <f t="shared" si="0"/>
+        <v>1.3436720763436725E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>62</v>
       </c>
@@ -2535,8 +2742,12 @@
       <c r="G38" s="1">
         <v>24522.015368750002</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H38">
+        <f t="shared" si="0"/>
+        <v>1.3436720763436725E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>51</v>
       </c>
@@ -2558,8 +2769,12 @@
       <c r="G39" s="1">
         <v>65146.784099999997</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H39">
+        <f t="shared" si="0"/>
+        <v>3.5696868035696876E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>56</v>
       </c>
@@ -2581,8 +2796,12 @@
       <c r="G40" s="1">
         <v>52558.355675000006</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H40">
+        <f t="shared" si="0"/>
+        <v>2.8799099028799107E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>38</v>
       </c>
@@ -2603,6 +2822,10 @@
       </c>
       <c r="G41" s="1">
         <v>119644.90854999999</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="0"/>
+        <v>6.5558854065558864E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>